<commit_message>
Generate Self Employed packages from app/data and app/templates
Triggered by: 28bfa156c60e2e30f6dcc393ab5f596e6c646f55
</commit_message>
<xml_diff>
--- a/examples/se-latest/Financialaccounts.xlsx
+++ b/examples/se-latest/Financialaccounts.xlsx
@@ -208,7 +208,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="799" uniqueCount="439">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="800" uniqueCount="440">
   <si>
     <r>
       <rPr>
@@ -1984,6 +1984,9 @@
   </si>
   <si>
     <t xml:space="preserve">Personal allowance taper threshold</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Special rate writing down allowance</t>
   </si>
   <si>
     <t xml:space="preserve">Basic rate applicable on taxable income up to higher rate</t>
@@ -4392,7 +4395,7 @@
       <sheetData sheetId="0">
         <row r="1">
           <cell r="I1">
-            <v>13740</v>
+            <v>17740</v>
           </cell>
         </row>
         <row r="1">
@@ -4403,7 +4406,7 @@
             <v>3360</v>
           </cell>
           <cell r="S1">
-            <v>20640</v>
+            <v>29100</v>
           </cell>
         </row>
         <row r="1">
@@ -4421,6 +4424,11 @@
           </cell>
           <cell r="Z1">
             <v>0</v>
+          </cell>
+        </row>
+        <row r="1">
+          <cell r="AC1">
+            <v>540</v>
           </cell>
         </row>
       </sheetData>
@@ -7774,7 +7782,9 @@
       <c r="N50" s="40" t="s">
         <v>33</v>
       </c>
-      <c r="O50" s="41"/>
+      <c r="O50" s="41" t="n">
+        <v>640</v>
+      </c>
       <c r="P50" s="41"/>
       <c r="Q50" s="41"/>
       <c r="R50" s="42" t="s">
@@ -8172,13 +8182,17 @@
         <v>46173</v>
       </c>
       <c r="C6" s="63"/>
-      <c r="D6" s="63"/>
+      <c r="D6" s="63" t="s">
+        <v>405</v>
+      </c>
       <c r="E6" s="63"/>
       <c r="F6" s="63"/>
-      <c r="G6" s="353"/>
+      <c r="G6" s="357" t="n">
+        <v>0.06</v>
+      </c>
       <c r="H6" s="63"/>
       <c r="I6" s="356" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="J6" s="356"/>
       <c r="K6" s="356"/>
@@ -8188,7 +8202,7 @@
         <v>0.2</v>
       </c>
       <c r="O6" s="353" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8198,14 +8212,14 @@
       </c>
       <c r="C7" s="63"/>
       <c r="D7" s="356" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="E7" s="356"/>
       <c r="F7" s="356"/>
       <c r="G7" s="353"/>
       <c r="H7" s="63"/>
       <c r="I7" s="356" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="J7" s="356"/>
       <c r="K7" s="356"/>
@@ -8215,7 +8229,7 @@
         <v>0.4</v>
       </c>
       <c r="O7" s="353" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8230,7 +8244,7 @@
       <c r="G8" s="359"/>
       <c r="H8" s="63"/>
       <c r="I8" s="356" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="J8" s="356"/>
       <c r="K8" s="356"/>
@@ -8240,7 +8254,7 @@
         <v>0.45</v>
       </c>
       <c r="O8" s="353" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8255,18 +8269,18 @@
       <c r="G9" s="353"/>
       <c r="H9" s="63"/>
       <c r="I9" s="356" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="J9" s="356"/>
       <c r="K9" s="356"/>
       <c r="L9" s="360" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="M9" s="360" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="N9" s="361" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="O9" s="353"/>
     </row>
@@ -8296,16 +8310,16 @@
       </c>
       <c r="C11" s="63"/>
       <c r="D11" s="349" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="E11" s="349"/>
       <c r="F11" s="349"/>
       <c r="G11" s="353" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="H11" s="63"/>
       <c r="I11" s="63" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="J11" s="63"/>
       <c r="K11" s="362" t="n">
@@ -8335,7 +8349,7 @@
       <c r="G12" s="353"/>
       <c r="H12" s="63"/>
       <c r="I12" s="63" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="J12" s="63"/>
       <c r="K12" s="362" t="n">
@@ -8357,7 +8371,7 @@
       </c>
       <c r="C13" s="63"/>
       <c r="D13" s="356" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="E13" s="356"/>
       <c r="F13" s="356"/>
@@ -8366,7 +8380,7 @@
       </c>
       <c r="H13" s="63"/>
       <c r="I13" s="63" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="J13" s="63"/>
       <c r="K13" s="362" t="n">
@@ -8388,7 +8402,7 @@
       </c>
       <c r="C14" s="63"/>
       <c r="D14" s="356" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="E14" s="356"/>
       <c r="F14" s="356"/>
@@ -8397,7 +8411,7 @@
       </c>
       <c r="H14" s="63"/>
       <c r="I14" s="349" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="J14" s="349"/>
       <c r="K14" s="349"/>
@@ -8416,7 +8430,7 @@
       </c>
       <c r="C15" s="63"/>
       <c r="D15" s="356" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="E15" s="356"/>
       <c r="F15" s="356"/>
@@ -8439,7 +8453,7 @@
       </c>
       <c r="C16" s="63"/>
       <c r="D16" s="356" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="E16" s="356"/>
       <c r="F16" s="356"/>
@@ -8448,7 +8462,7 @@
       </c>
       <c r="H16" s="63"/>
       <c r="I16" s="356" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="J16" s="356"/>
       <c r="K16" s="356"/>
@@ -8456,7 +8470,7 @@
         <v>3.65</v>
       </c>
       <c r="M16" s="63" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="N16" s="359" t="n">
         <v>7105</v>
@@ -8472,7 +8486,7 @@
       </c>
       <c r="C17" s="63"/>
       <c r="D17" s="356" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="E17" s="356"/>
       <c r="F17" s="356"/>
@@ -8514,24 +8528,24 @@
       </c>
       <c r="C19" s="63"/>
       <c r="D19" s="349" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="E19" s="349"/>
       <c r="F19" s="353" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="G19" s="353" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="H19" s="63"/>
       <c r="I19" s="365" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="J19" s="365"/>
       <c r="K19" s="365"/>
       <c r="L19" s="63"/>
       <c r="M19" s="366" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="N19" s="63"/>
       <c r="O19" s="63"/>
@@ -8568,7 +8582,7 @@
       </c>
       <c r="C21" s="63"/>
       <c r="D21" s="356" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="E21" s="356"/>
       <c r="F21" s="359" t="n">
@@ -8593,7 +8607,7 @@
       </c>
       <c r="C22" s="63"/>
       <c r="D22" s="63" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="E22" s="63"/>
       <c r="F22" s="359" t="n">
@@ -8604,13 +8618,13 @@
       </c>
       <c r="H22" s="63"/>
       <c r="I22" s="365" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="J22" s="365"/>
       <c r="K22" s="365"/>
       <c r="L22" s="63"/>
       <c r="M22" s="366" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="N22" s="63"/>
       <c r="O22" s="63"/>
@@ -8618,7 +8632,7 @@
     <row r="23" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="63"/>
       <c r="B23" s="355" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="C23" s="63"/>
       <c r="D23" s="63"/>
@@ -8643,11 +8657,11 @@
     <row r="24" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="63"/>
       <c r="B24" s="355" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C24" s="63"/>
       <c r="D24" s="349" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="E24" s="349"/>
       <c r="F24" s="63"/>
@@ -8685,7 +8699,7 @@
       <c r="B26" s="369"/>
       <c r="C26" s="63"/>
       <c r="D26" s="356" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="E26" s="356"/>
       <c r="F26" s="359" t="n">
@@ -8706,7 +8720,7 @@
       <c r="B27" s="369"/>
       <c r="C27" s="63"/>
       <c r="D27" s="63" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="E27" s="63"/>
       <c r="F27" s="357" t="n">
@@ -11175,8 +11189,8 @@
         <v>33</v>
       </c>
       <c r="O80" s="98" t="n">
-        <f aca="false">IF(([1]Schedule!$R$1+[1]Schedule!$Y$1)&gt;0,[1]Schedule!$R$1+[1]Schedule!$Y$1,0)</f>
-        <v>11500</v>
+        <f aca="false">IF(([1]Schedule!$R$1+[1]Schedule!$Y$1+[1]Schedule!$AC$1)&gt;0,[1]Schedule!$R$1+[1]Schedule!$Y$1+[1]Schedule!$AC$1,0)</f>
+        <v>12040</v>
       </c>
       <c r="P80" s="98"/>
       <c r="Q80" s="98"/>
@@ -11578,7 +11592,7 @@
       </c>
       <c r="D94" s="98" t="n">
         <f aca="false">'Business Details'!O50</f>
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="E94" s="98"/>
       <c r="F94" s="98"/>
@@ -11737,7 +11751,7 @@
       </c>
       <c r="D99" s="98" t="n">
         <f aca="false">IF((D71+O85+D94-O71-D80-D85-O80)&gt;0,D71+O85+D94-O71-D80-D85-O80,0)</f>
-        <v>128469.475166666</v>
+        <v>128569.475166666</v>
       </c>
       <c r="E99" s="98"/>
       <c r="F99" s="98"/>
@@ -11950,7 +11964,7 @@
       </c>
       <c r="D106" s="98" t="n">
         <f aca="false">IF((D99+O99-O94)&gt;0,D99+O99-O94,0)</f>
-        <v>130552.8085</v>
+        <v>130652.8085</v>
       </c>
       <c r="E106" s="98"/>
       <c r="F106" s="98"/>
@@ -16050,7 +16064,7 @@
       </c>
       <c r="D114" s="98" t="n">
         <f aca="false">'Profit &amp; Loss Account'!B33+'Profit &amp; Loss Account'!B34</f>
-        <v>13912</v>
+        <v>17912</v>
       </c>
       <c r="E114" s="98"/>
       <c r="F114" s="98"/>
@@ -16072,7 +16086,7 @@
       </c>
       <c r="O114" s="98" t="n">
         <f aca="false">'Profit &amp; Loss Account'!B34</f>
-        <v>13740</v>
+        <v>17740</v>
       </c>
       <c r="P114" s="98"/>
       <c r="Q114" s="98"/>
@@ -16308,7 +16322,7 @@
       </c>
       <c r="D122" s="98" t="n">
         <f aca="false">'Profit &amp; Loss Account'!B17+'Profit &amp; Loss Account'!B35</f>
-        <v>169801.983333333</v>
+        <v>173801.983333333</v>
       </c>
       <c r="E122" s="98"/>
       <c r="F122" s="98"/>
@@ -16330,7 +16344,7 @@
       </c>
       <c r="O122" s="98" t="n">
         <f aca="false">O66+O70+O74+O78+O82+O86+O90+O94+O98+O102+O106+O110+O114+O118</f>
-        <v>23071.4585</v>
+        <v>27071.4585</v>
       </c>
       <c r="P122" s="98"/>
       <c r="Q122" s="98"/>
@@ -16519,7 +16533,7 @@
       </c>
       <c r="D129" s="98" t="n">
         <f aca="false">IF((D55+O55-D122)&gt;=0,D55+O55-D122,0)</f>
-        <v>169398.016666666</v>
+        <v>165398.016666666</v>
       </c>
       <c r="E129" s="98"/>
       <c r="F129" s="98"/>
@@ -17065,7 +17079,10 @@
       <c r="C147" s="97" t="s">
         <v>33</v>
       </c>
-      <c r="D147" s="98"/>
+      <c r="D147" s="98" t="n">
+        <f aca="false">[1]Schedule!$AC$1</f>
+        <v>540</v>
+      </c>
       <c r="E147" s="98"/>
       <c r="F147" s="98"/>
       <c r="G147" s="99" t="s">
@@ -17298,7 +17315,7 @@
       </c>
       <c r="O154" s="98" t="n">
         <f aca="false">D139+D144+D147+D152+D156+D160+O139+O144+O149</f>
-        <v>64000</v>
+        <v>68840</v>
       </c>
       <c r="P154" s="98"/>
       <c r="Q154" s="98"/>
@@ -17346,7 +17363,9 @@
       <c r="C156" s="97" t="s">
         <v>33</v>
       </c>
-      <c r="D156" s="98"/>
+      <c r="D156" s="98" t="n">
+        <v>2500</v>
+      </c>
       <c r="E156" s="98"/>
       <c r="F156" s="98"/>
       <c r="G156" s="99" t="s">
@@ -17466,7 +17485,9 @@
       <c r="C160" s="97" t="s">
         <v>33</v>
       </c>
-      <c r="D160" s="98"/>
+      <c r="D160" s="98" t="n">
+        <v>1800</v>
+      </c>
       <c r="E160" s="98"/>
       <c r="F160" s="98"/>
       <c r="G160" s="99" t="s">
@@ -17728,7 +17749,7 @@
       </c>
       <c r="D169" s="98" t="n">
         <f aca="false">'Business Details'!O50</f>
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="E169" s="98"/>
       <c r="F169" s="98"/>
@@ -17750,7 +17771,7 @@
       </c>
       <c r="O169" s="98" t="n">
         <f aca="false">O154+D179</f>
-        <v>64000</v>
+        <v>69190</v>
       </c>
       <c r="P169" s="98"/>
       <c r="Q169" s="98"/>
@@ -17887,7 +17908,7 @@
       </c>
       <c r="D174" s="98" t="n">
         <f aca="false">O122+O160+D169</f>
-        <v>23071.4585</v>
+        <v>27711.4585</v>
       </c>
       <c r="E174" s="98"/>
       <c r="F174" s="98"/>
@@ -17909,7 +17930,7 @@
       </c>
       <c r="O174" s="98" t="n">
         <f aca="false">IF((D129+D174-O169)&gt;0,(D129+D174-O169),IF((-O129+D174-O169)&gt;0,(-O129+D174-O169),0))</f>
-        <v>128469.475166666</v>
+        <v>123919.475166666</v>
       </c>
       <c r="P174" s="98"/>
       <c r="Q174" s="98"/>
@@ -18044,7 +18065,9 @@
       <c r="C179" s="97" t="s">
         <v>33</v>
       </c>
-      <c r="D179" s="98"/>
+      <c r="D179" s="98" t="n">
+        <v>350</v>
+      </c>
       <c r="E179" s="98"/>
       <c r="F179" s="98"/>
       <c r="G179" s="99" t="s">
@@ -18498,7 +18521,7 @@
       </c>
       <c r="O194" s="98" t="n">
         <f aca="false">O174</f>
-        <v>128469.475166666</v>
+        <v>123919.475166666</v>
       </c>
       <c r="P194" s="98"/>
       <c r="Q194" s="98"/>
@@ -18952,7 +18975,9 @@
       <c r="C210" s="97" t="s">
         <v>33</v>
       </c>
-      <c r="D210" s="98"/>
+      <c r="D210" s="98" t="n">
+        <v>90</v>
+      </c>
       <c r="E210" s="98"/>
       <c r="F210" s="98"/>
       <c r="G210" s="99" t="s">
@@ -18973,7 +18998,7 @@
       </c>
       <c r="O210" s="98" t="n">
         <f aca="false">O194-O199+O204</f>
-        <v>130552.8085</v>
+        <v>126002.8085</v>
       </c>
       <c r="P210" s="98"/>
       <c r="Q210" s="98"/>
@@ -19219,7 +19244,7 @@
       </c>
       <c r="D219" s="98" t="n">
         <f aca="false">O179+E197+D210+P190</f>
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="E219" s="98"/>
       <c r="F219" s="98"/>
@@ -19397,7 +19422,7 @@
       </c>
       <c r="O224" s="98" t="n">
         <f aca="false">D219</f>
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="P224" s="98"/>
       <c r="Q224" s="98"/>
@@ -24022,55 +24047,55 @@
       </c>
       <c r="B34" s="171" t="n">
         <f aca="false">SUM(C34:N34)</f>
-        <v>13740</v>
+        <v>17740</v>
       </c>
       <c r="C34" s="172" t="n">
         <f aca="false">([1]Schedule!$I$1)/12</f>
-        <v>1145</v>
+        <v>1478.33333333333</v>
       </c>
       <c r="D34" s="172" t="n">
         <f aca="false">([1]Schedule!$I$1)/12</f>
-        <v>1145</v>
+        <v>1478.33333333333</v>
       </c>
       <c r="E34" s="173" t="n">
         <f aca="false">([1]Schedule!$I$1)/12</f>
-        <v>1145</v>
+        <v>1478.33333333333</v>
       </c>
       <c r="F34" s="172" t="n">
         <f aca="false">([1]Schedule!$I$1)/12</f>
-        <v>1145</v>
+        <v>1478.33333333333</v>
       </c>
       <c r="G34" s="172" t="n">
         <f aca="false">([1]Schedule!$I$1)/12</f>
-        <v>1145</v>
+        <v>1478.33333333333</v>
       </c>
       <c r="H34" s="173" t="n">
         <f aca="false">([1]Schedule!$I$1)/12</f>
-        <v>1145</v>
+        <v>1478.33333333333</v>
       </c>
       <c r="I34" s="172" t="n">
         <f aca="false">([1]Schedule!$I$1)/12</f>
-        <v>1145</v>
+        <v>1478.33333333333</v>
       </c>
       <c r="J34" s="172" t="n">
         <f aca="false">([1]Schedule!$I$1)/12</f>
-        <v>1145</v>
+        <v>1478.33333333333</v>
       </c>
       <c r="K34" s="173" t="n">
         <f aca="false">([1]Schedule!$I$1)/12</f>
-        <v>1145</v>
+        <v>1478.33333333333</v>
       </c>
       <c r="L34" s="172" t="n">
         <f aca="false">([1]Schedule!$I$1)/12</f>
-        <v>1145</v>
+        <v>1478.33333333333</v>
       </c>
       <c r="M34" s="172" t="n">
         <f aca="false">([1]Schedule!$I$1)/12</f>
-        <v>1145</v>
+        <v>1478.33333333333</v>
       </c>
       <c r="N34" s="172" t="n">
         <f aca="false">([1]Schedule!$I$1)/12</f>
-        <v>1145</v>
+        <v>1478.33333333333</v>
       </c>
       <c r="O34" s="165"/>
     </row>
@@ -24080,55 +24105,55 @@
       </c>
       <c r="B35" s="171" t="n">
         <f aca="false">SUM(B21:B34)</f>
-        <v>149665.316666667</v>
+        <v>153665.316666667</v>
       </c>
       <c r="C35" s="171" t="n">
         <f aca="false">SUM(C21:C34)</f>
-        <v>12012.7833333333</v>
+        <v>12346.1166666667</v>
       </c>
       <c r="D35" s="171" t="n">
         <f aca="false">SUM(D21:D34)</f>
-        <v>11323.5333333333</v>
+        <v>11656.8666666667</v>
       </c>
       <c r="E35" s="171" t="n">
         <f aca="false">SUM(E21:E34)</f>
-        <v>13592.8666666667</v>
+        <v>13926.2</v>
       </c>
       <c r="F35" s="175" t="n">
         <f aca="false">SUM(F21:F34)</f>
-        <v>13829.7833333333</v>
+        <v>14163.1166666667</v>
       </c>
       <c r="G35" s="171" t="n">
         <f aca="false">SUM(G21:G34)</f>
-        <v>11766.1166666667</v>
+        <v>12099.45</v>
       </c>
       <c r="H35" s="171" t="n">
         <f aca="false">SUM(H21:H34)</f>
-        <v>13242.8666666667</v>
+        <v>13576.2</v>
       </c>
       <c r="I35" s="175" t="n">
         <f aca="false">SUM(I21:I34)</f>
-        <v>13692.2833333333</v>
+        <v>14025.6166666667</v>
       </c>
       <c r="J35" s="171" t="n">
         <f aca="false">SUM(J21:J34)</f>
-        <v>10880.5333333333</v>
+        <v>11213.8666666667</v>
       </c>
       <c r="K35" s="171" t="n">
         <f aca="false">SUM(K21:K34)</f>
-        <v>15898.5333333333</v>
+        <v>16231.8666666667</v>
       </c>
       <c r="L35" s="175" t="n">
         <f aca="false">SUM(L21:L34)</f>
-        <v>11392.7833333333</v>
+        <v>11726.1166666667</v>
       </c>
       <c r="M35" s="171" t="n">
         <f aca="false">SUM(M21:M34)</f>
-        <v>11066.0333333333</v>
+        <v>11399.3666666667</v>
       </c>
       <c r="N35" s="171" t="n">
         <f aca="false">SUM(N21:N34)</f>
-        <v>10967.2</v>
+        <v>11300.5333333333</v>
       </c>
       <c r="O35" s="165"/>
     </row>
@@ -24155,55 +24180,55 @@
       </c>
       <c r="B37" s="171" t="n">
         <f aca="false">B19-B35</f>
-        <v>171481.35</v>
+        <v>167481.35</v>
       </c>
       <c r="C37" s="171" t="n">
         <f aca="false">C19-C35</f>
-        <v>15083.05</v>
+        <v>14749.7166666666</v>
       </c>
       <c r="D37" s="171" t="n">
         <f aca="false">D19-D35</f>
-        <v>15102.3</v>
+        <v>14768.9666666666</v>
       </c>
       <c r="E37" s="171" t="n">
         <f aca="false">E19-E35</f>
-        <v>11036.3</v>
+        <v>10702.9666666666</v>
       </c>
       <c r="F37" s="175" t="n">
         <f aca="false">F19-F35</f>
-        <v>13096.05</v>
+        <v>12762.7166666666</v>
       </c>
       <c r="G37" s="171" t="n">
         <f aca="false">G19-G35</f>
-        <v>17563.05</v>
+        <v>17229.7166666666</v>
       </c>
       <c r="H37" s="171" t="n">
         <f aca="false">H19-H35</f>
-        <v>14182.9666666666</v>
+        <v>13849.6333333333</v>
       </c>
       <c r="I37" s="175" t="n">
         <f aca="false">I19-I35</f>
-        <v>15303.55</v>
+        <v>14970.2166666666</v>
       </c>
       <c r="J37" s="171" t="n">
         <f aca="false">J19-J35</f>
-        <v>15145.3</v>
+        <v>14811.9666666666</v>
       </c>
       <c r="K37" s="171" t="n">
         <f aca="false">K19-K35</f>
-        <v>10797.3</v>
+        <v>10463.9666666666</v>
       </c>
       <c r="L37" s="175" t="n">
         <f aca="false">L19-L35</f>
-        <v>17283.05</v>
+        <v>16949.7166666666</v>
       </c>
       <c r="M37" s="171" t="n">
         <f aca="false">M19-M35</f>
-        <v>16479.8</v>
+        <v>16146.4666666666</v>
       </c>
       <c r="N37" s="171" t="n">
         <f aca="false">N19-N35</f>
-        <v>10408.6333333333</v>
+        <v>10075.3</v>
       </c>
       <c r="O37" s="165"/>
     </row>
@@ -24271,55 +24296,55 @@
       </c>
       <c r="B39" s="171" t="n">
         <f aca="false">B37+B38</f>
-        <v>171481.35</v>
+        <v>167481.35</v>
       </c>
       <c r="C39" s="171" t="n">
         <f aca="false">C37+C38</f>
-        <v>15083.05</v>
+        <v>14749.7166666666</v>
       </c>
       <c r="D39" s="171" t="n">
         <f aca="false">D37+D38</f>
-        <v>15102.3</v>
+        <v>14768.9666666666</v>
       </c>
       <c r="E39" s="171" t="n">
         <f aca="false">E37+E38</f>
-        <v>11036.3</v>
+        <v>10702.9666666666</v>
       </c>
       <c r="F39" s="175" t="n">
         <f aca="false">F37+F38</f>
-        <v>13096.05</v>
+        <v>12762.7166666666</v>
       </c>
       <c r="G39" s="171" t="n">
         <f aca="false">G37+G38</f>
-        <v>17563.05</v>
+        <v>17229.7166666666</v>
       </c>
       <c r="H39" s="171" t="n">
         <f aca="false">H37+H38</f>
-        <v>14182.9666666666</v>
+        <v>13849.6333333333</v>
       </c>
       <c r="I39" s="175" t="n">
         <f aca="false">I37+I38</f>
-        <v>15303.55</v>
+        <v>14970.2166666666</v>
       </c>
       <c r="J39" s="171" t="n">
         <f aca="false">J37+J38</f>
-        <v>15145.3</v>
+        <v>14811.9666666666</v>
       </c>
       <c r="K39" s="171" t="n">
         <f aca="false">K37+K38</f>
-        <v>10797.3</v>
+        <v>10463.9666666666</v>
       </c>
       <c r="L39" s="175" t="n">
         <f aca="false">L37+L38</f>
-        <v>17283.05</v>
+        <v>16949.7166666666</v>
       </c>
       <c r="M39" s="171" t="n">
         <f aca="false">M37+M38</f>
-        <v>16479.8</v>
+        <v>16146.4666666666</v>
       </c>
       <c r="N39" s="171" t="n">
         <f aca="false">N37+N38</f>
-        <v>10408.6333333333</v>
+        <v>10075.3</v>
       </c>
       <c r="O39" s="165"/>
     </row>
@@ -24481,55 +24506,55 @@
       </c>
       <c r="B44" s="178" t="n">
         <f aca="false">SUM(C44:N44)</f>
-        <v>43952.4769999998</v>
+        <v>43617.6769999997</v>
       </c>
       <c r="C44" s="178" t="n">
         <f aca="false">IF(C9&gt;0,'Profit Forecast'!C$46/12,0)</f>
-        <v>3662.70641666665</v>
+        <v>3634.80641666665</v>
       </c>
       <c r="D44" s="178" t="n">
         <f aca="false">IF(D9&gt;0,'Profit Forecast'!C$46/12,0)</f>
-        <v>3662.70641666665</v>
+        <v>3634.80641666665</v>
       </c>
       <c r="E44" s="178" t="n">
         <f aca="false">IF(E9&gt;0,'Profit Forecast'!C$46/12,0)</f>
-        <v>3662.70641666665</v>
+        <v>3634.80641666665</v>
       </c>
       <c r="F44" s="178" t="n">
         <f aca="false">IF(F9&gt;0,'Profit Forecast'!C$46/12,0)</f>
-        <v>3662.70641666665</v>
+        <v>3634.80641666665</v>
       </c>
       <c r="G44" s="178" t="n">
         <f aca="false">IF(G9&gt;0,'Profit Forecast'!C$46/12,0)</f>
-        <v>3662.70641666665</v>
+        <v>3634.80641666665</v>
       </c>
       <c r="H44" s="178" t="n">
         <f aca="false">IF(H9&gt;0,'Profit Forecast'!C$46/12,0)</f>
-        <v>3662.70641666665</v>
+        <v>3634.80641666665</v>
       </c>
       <c r="I44" s="178" t="n">
         <f aca="false">IF(I9&gt;0,'Profit Forecast'!C$46/12,0)</f>
-        <v>3662.70641666665</v>
+        <v>3634.80641666665</v>
       </c>
       <c r="J44" s="178" t="n">
         <f aca="false">IF(J9&gt;0,'Profit Forecast'!C$46/12,0)</f>
-        <v>3662.70641666665</v>
+        <v>3634.80641666665</v>
       </c>
       <c r="K44" s="178" t="n">
         <f aca="false">IF(K9&gt;0,'Profit Forecast'!C$46/12,0)</f>
-        <v>3662.70641666665</v>
+        <v>3634.80641666665</v>
       </c>
       <c r="L44" s="178" t="n">
         <f aca="false">IF(L9&gt;0,'Profit Forecast'!C$46/12,0)</f>
-        <v>3662.70641666665</v>
+        <v>3634.80641666665</v>
       </c>
       <c r="M44" s="178" t="n">
         <f aca="false">IF(M9&gt;0,'Profit Forecast'!C$46/12,0)</f>
-        <v>3662.70641666665</v>
+        <v>3634.80641666665</v>
       </c>
       <c r="N44" s="178" t="n">
         <f aca="false">IF(N9&gt;0,'Profit Forecast'!C$46/12,0)</f>
-        <v>3662.70641666665</v>
+        <v>3634.80641666665</v>
       </c>
       <c r="O44" s="165"/>
     </row>
@@ -24539,55 +24564,55 @@
       </c>
       <c r="B45" s="190" t="n">
         <f aca="false">SUM(C45:N45)</f>
-        <v>100528.873</v>
+        <v>96863.6729999998</v>
       </c>
       <c r="C45" s="191" t="n">
         <f aca="false">C39-C42-C44</f>
-        <v>10420.3435833333</v>
+        <v>10114.91025</v>
       </c>
       <c r="D45" s="192" t="n">
         <f aca="false">D39-D42-D44</f>
-        <v>10439.5935833333</v>
+        <v>10134.16025</v>
       </c>
       <c r="E45" s="192" t="n">
         <f aca="false">E39-E42-E44</f>
-        <v>6373.59358333332</v>
+        <v>6068.16024999998</v>
       </c>
       <c r="F45" s="192" t="n">
         <f aca="false">F39-F42-F44</f>
-        <v>5433.34358333332</v>
+        <v>5127.91024999999</v>
       </c>
       <c r="G45" s="192" t="n">
         <f aca="false">G39-G42-G44</f>
-        <v>12900.3435833333</v>
+        <v>12594.91025</v>
       </c>
       <c r="H45" s="192" t="n">
         <f aca="false">H39-H42-H44</f>
-        <v>9520.26024999999</v>
+        <v>9214.82691666666</v>
       </c>
       <c r="I45" s="192" t="n">
         <f aca="false">I39-I42-I44</f>
-        <v>7640.84358333332</v>
+        <v>7335.41024999999</v>
       </c>
       <c r="J45" s="192" t="n">
         <f aca="false">J39-J42-J44</f>
-        <v>10482.5935833333</v>
+        <v>10177.16025</v>
       </c>
       <c r="K45" s="192" t="n">
         <f aca="false">K39-K42-K44</f>
-        <v>6134.59358333332</v>
+        <v>5829.16024999998</v>
       </c>
       <c r="L45" s="192" t="n">
         <f aca="false">L39-L42-L44</f>
-        <v>9620.34358333332</v>
+        <v>9314.91024999999</v>
       </c>
       <c r="M45" s="192" t="n">
         <f aca="false">M39-M42-M44</f>
-        <v>11817.0935833333</v>
+        <v>11511.66025</v>
       </c>
       <c r="N45" s="192" t="n">
         <f aca="false">N39-N42-N44</f>
-        <v>-254.073083333347</v>
+        <v>-559.50641666668</v>
       </c>
       <c r="O45" s="165"/>
     </row>
@@ -25339,23 +25364,23 @@
       </c>
       <c r="C26" s="201" t="n">
         <f aca="false">SUM('Profit &amp; Loss Account'!C33:E34)</f>
-        <v>3478</v>
+        <v>4478</v>
       </c>
       <c r="D26" s="201" t="n">
         <f aca="false">SUM('Profit &amp; Loss Account'!F33:H34)</f>
-        <v>3478</v>
+        <v>4478</v>
       </c>
       <c r="E26" s="201" t="n">
         <f aca="false">SUM('Profit &amp; Loss Account'!I33:K34)</f>
-        <v>3478</v>
+        <v>4478</v>
       </c>
       <c r="F26" s="201" t="n">
         <f aca="false">SUM('Profit &amp; Loss Account'!L33:N34)</f>
-        <v>3478</v>
+        <v>4478</v>
       </c>
       <c r="G26" s="201" t="n">
         <f aca="false">SUM(C26:F26)</f>
-        <v>13912</v>
+        <v>17912</v>
       </c>
       <c r="H26" s="196"/>
       <c r="I26" s="196"/>
@@ -25389,23 +25414,23 @@
       </c>
       <c r="C29" s="204" t="n">
         <f aca="false">SUM(C7,C12,C13,C14,C15,C16,C17,C18,C19,C20,C21,C22,C24,C26)</f>
-        <v>43378.35</v>
+        <v>44378.35</v>
       </c>
       <c r="D29" s="204" t="n">
         <f aca="false">SUM(D7,D12,D13,D14,D15,D16,D17,D18,D19,D20,D21,D22,D24,D26)</f>
-        <v>41441.2666666667</v>
+        <v>42441.2666666667</v>
       </c>
       <c r="E29" s="204" t="n">
         <f aca="false">SUM(E7,E12,E13,E14,E15,E16,E17,E18,E19,E20,E21,E22,E24,E26)</f>
-        <v>45153.85</v>
+        <v>46153.85</v>
       </c>
       <c r="F29" s="204" t="n">
         <f aca="false">SUM(F7,F12,F13,F14,F15,F16,F17,F18,F19,F20,F21,F22,F24,F26)</f>
-        <v>39828.5166666667</v>
+        <v>40828.5166666667</v>
       </c>
       <c r="G29" s="204" t="n">
         <f aca="false">SUM(G7,G12,G13,G14,G15,G16,G17,G18,G19,G20,G21,G22,G24,G26)</f>
-        <v>169801.983333333</v>
+        <v>173801.983333333</v>
       </c>
       <c r="H29" s="205"/>
       <c r="I29" s="196"/>
@@ -25899,23 +25924,23 @@
       </c>
       <c r="C49" s="201" t="n">
         <f aca="false">SUM('Profit &amp; Loss Account'!C34:E34)</f>
-        <v>3435</v>
+        <v>4435</v>
       </c>
       <c r="D49" s="201" t="n">
         <f aca="false">SUM('Profit &amp; Loss Account'!F34:H34)</f>
-        <v>3435</v>
+        <v>4435</v>
       </c>
       <c r="E49" s="201" t="n">
         <f aca="false">SUM('Profit &amp; Loss Account'!I34:K34)</f>
-        <v>3435</v>
+        <v>4435</v>
       </c>
       <c r="F49" s="201" t="n">
         <f aca="false">SUM('Profit &amp; Loss Account'!L34:N34)</f>
-        <v>3435</v>
+        <v>4435</v>
       </c>
       <c r="G49" s="201" t="n">
         <f aca="false">SUM(C49:F49)</f>
-        <v>13740</v>
+        <v>17740</v>
       </c>
       <c r="H49" s="196" t="s">
         <v>322</v>
@@ -26061,7 +26086,7 @@
       <c r="D5" s="223"/>
       <c r="E5" s="224" t="n">
         <f aca="false">'SE Full'!O210</f>
-        <v>130552.8085</v>
+        <v>126002.8085</v>
       </c>
       <c r="F5" s="215"/>
       <c r="G5" s="219"/>
@@ -26094,7 +26119,7 @@
       <c r="D7" s="223"/>
       <c r="E7" s="224" t="n">
         <f aca="false">IF((E5&gt;E6),(E5-E6),0)</f>
-        <v>130552.8085</v>
+        <v>126002.8085</v>
       </c>
       <c r="F7" s="215"/>
       <c r="G7" s="219"/>
@@ -26158,7 +26183,7 @@
       </c>
       <c r="E10" s="214" t="n">
         <f aca="false">IF(E7&gt;C10,(E7-C10)*D10,0)</f>
-        <v>2435.76382499982</v>
+        <v>388.263824999816</v>
       </c>
       <c r="F10" s="215"/>
       <c r="G10" s="219"/>
@@ -26173,7 +26198,7 @@
       <c r="D11" s="231"/>
       <c r="E11" s="232" t="n">
         <f aca="false">SUM(E8:E10)</f>
-        <v>44951.7638249998</v>
+        <v>42904.2638249998</v>
       </c>
       <c r="F11" s="233"/>
       <c r="G11" s="234"/>
@@ -26249,7 +26274,7 @@
       </c>
       <c r="E16" s="241" t="n">
         <f aca="false">IF((E5&gt;Admin!N$23),((E5-Admin!N$23)*D16),0)</f>
-        <v>1605.65616999999</v>
+        <v>1514.65616999999</v>
       </c>
       <c r="F16" s="215"/>
       <c r="G16" s="234"/>
@@ -26274,7 +26299,7 @@
       <c r="D18" s="238"/>
       <c r="E18" s="232" t="n">
         <f aca="false">SUM(E11:E17)</f>
-        <v>48819.4199949998</v>
+        <v>46680.9199949998</v>
       </c>
       <c r="F18" s="215"/>
       <c r="G18" s="219"/>
@@ -26356,7 +26381,7 @@
       </c>
       <c r="E25" s="241" t="n">
         <f aca="false">E18</f>
-        <v>48819.4199949998</v>
+        <v>46680.9199949998</v>
       </c>
       <c r="F25" s="215"/>
       <c r="G25" s="219"/>
@@ -26373,7 +26398,7 @@
       </c>
       <c r="E26" s="224" t="n">
         <f aca="false">E25/2</f>
-        <v>24409.7099974999</v>
+        <v>23340.4599974999</v>
       </c>
       <c r="F26" s="215"/>
       <c r="G26" s="219"/>
@@ -26390,7 +26415,7 @@
       </c>
       <c r="E27" s="224" t="n">
         <f aca="false">E25/2</f>
-        <v>24409.7099974999</v>
+        <v>23340.4599974999</v>
       </c>
       <c r="F27" s="215"/>
       <c r="G27" s="219"/>
@@ -29306,55 +29331,55 @@
       </c>
       <c r="C13" s="171" t="n">
         <f aca="false">SUM(D13:O13)</f>
-        <v>149665.316666667</v>
+        <v>153665.316666667</v>
       </c>
       <c r="D13" s="171" t="n">
         <f aca="false">'Profit &amp; Loss Account'!C35</f>
-        <v>12012.7833333333</v>
+        <v>12346.1166666667</v>
       </c>
       <c r="E13" s="171" t="n">
         <f aca="false">'Profit &amp; Loss Account'!D35</f>
-        <v>11323.5333333333</v>
+        <v>11656.8666666667</v>
       </c>
       <c r="F13" s="171" t="n">
         <f aca="false">'Profit &amp; Loss Account'!E35</f>
-        <v>13592.8666666667</v>
+        <v>13926.2</v>
       </c>
       <c r="G13" s="171" t="n">
         <f aca="false">'Profit &amp; Loss Account'!F35</f>
-        <v>13829.7833333333</v>
+        <v>14163.1166666667</v>
       </c>
       <c r="H13" s="171" t="n">
         <f aca="false">'Profit &amp; Loss Account'!G35</f>
-        <v>11766.1166666667</v>
+        <v>12099.45</v>
       </c>
       <c r="I13" s="171" t="n">
         <f aca="false">'Profit &amp; Loss Account'!H35</f>
-        <v>13242.8666666667</v>
+        <v>13576.2</v>
       </c>
       <c r="J13" s="171" t="n">
         <f aca="false">'Profit &amp; Loss Account'!I35</f>
-        <v>13692.2833333333</v>
+        <v>14025.6166666667</v>
       </c>
       <c r="K13" s="171" t="n">
         <f aca="false">'Profit &amp; Loss Account'!J35</f>
-        <v>10880.5333333333</v>
+        <v>11213.8666666667</v>
       </c>
       <c r="L13" s="171" t="n">
         <f aca="false">'Profit &amp; Loss Account'!K35</f>
-        <v>15898.5333333333</v>
+        <v>16231.8666666667</v>
       </c>
       <c r="M13" s="171" t="n">
         <f aca="false">'Profit &amp; Loss Account'!L35</f>
-        <v>11392.7833333333</v>
+        <v>11726.1166666667</v>
       </c>
       <c r="N13" s="171" t="n">
         <f aca="false">'Profit &amp; Loss Account'!M35</f>
-        <v>11066.0333333333</v>
+        <v>11399.3666666667</v>
       </c>
       <c r="O13" s="171" t="n">
         <f aca="false">'Profit &amp; Loss Account'!N35</f>
-        <v>10967.2</v>
+        <v>11300.5333333333</v>
       </c>
       <c r="P13" s="159"/>
     </row>
@@ -29383,55 +29408,55 @@
       </c>
       <c r="C15" s="171" t="n">
         <f aca="false">SUM(D15:O15)</f>
-        <v>171481.35</v>
+        <v>167481.35</v>
       </c>
       <c r="D15" s="171" t="n">
         <f aca="false">D11-D13</f>
-        <v>15083.05</v>
+        <v>14749.7166666666</v>
       </c>
       <c r="E15" s="171" t="n">
         <f aca="false">E11-E13</f>
-        <v>15102.3</v>
+        <v>14768.9666666666</v>
       </c>
       <c r="F15" s="171" t="n">
         <f aca="false">F11-F13</f>
-        <v>11036.3</v>
+        <v>10702.9666666666</v>
       </c>
       <c r="G15" s="171" t="n">
         <f aca="false">G11-G13</f>
-        <v>13096.05</v>
+        <v>12762.7166666666</v>
       </c>
       <c r="H15" s="171" t="n">
         <f aca="false">H11-H13</f>
-        <v>17563.05</v>
+        <v>17229.7166666666</v>
       </c>
       <c r="I15" s="171" t="n">
         <f aca="false">I11-I13</f>
-        <v>14182.9666666666</v>
+        <v>13849.6333333333</v>
       </c>
       <c r="J15" s="171" t="n">
         <f aca="false">J11-J13</f>
-        <v>15303.55</v>
+        <v>14970.2166666666</v>
       </c>
       <c r="K15" s="171" t="n">
         <f aca="false">K11-K13</f>
-        <v>15145.3</v>
+        <v>14811.9666666666</v>
       </c>
       <c r="L15" s="171" t="n">
         <f aca="false">L11-L13</f>
-        <v>10797.3</v>
+        <v>10463.9666666666</v>
       </c>
       <c r="M15" s="171" t="n">
         <f aca="false">M11-M13</f>
-        <v>17283.05</v>
+        <v>16949.7166666666</v>
       </c>
       <c r="N15" s="171" t="n">
         <f aca="false">N11-N13</f>
-        <v>16479.8</v>
+        <v>16146.4666666666</v>
       </c>
       <c r="O15" s="171" t="n">
         <f aca="false">O11-O13</f>
-        <v>10408.6333333333</v>
+        <v>10075.3</v>
       </c>
       <c r="P15" s="159"/>
     </row>
@@ -29501,55 +29526,55 @@
       </c>
       <c r="C17" s="171" t="n">
         <f aca="false">SUM(D17:O17)</f>
-        <v>171481.35</v>
+        <v>167481.35</v>
       </c>
       <c r="D17" s="171" t="n">
         <f aca="false">D15+D16</f>
-        <v>15083.05</v>
+        <v>14749.7166666666</v>
       </c>
       <c r="E17" s="171" t="n">
         <f aca="false">E15+E16</f>
-        <v>15102.3</v>
+        <v>14768.9666666666</v>
       </c>
       <c r="F17" s="171" t="n">
         <f aca="false">F15+F16</f>
-        <v>11036.3</v>
+        <v>10702.9666666666</v>
       </c>
       <c r="G17" s="171" t="n">
         <f aca="false">G15+G16</f>
-        <v>13096.05</v>
+        <v>12762.7166666666</v>
       </c>
       <c r="H17" s="171" t="n">
         <f aca="false">H15+H16</f>
-        <v>17563.05</v>
+        <v>17229.7166666666</v>
       </c>
       <c r="I17" s="171" t="n">
         <f aca="false">I15+I16</f>
-        <v>14182.9666666666</v>
+        <v>13849.6333333333</v>
       </c>
       <c r="J17" s="171" t="n">
         <f aca="false">J15+J16</f>
-        <v>15303.55</v>
+        <v>14970.2166666666</v>
       </c>
       <c r="K17" s="171" t="n">
         <f aca="false">K15+K16</f>
-        <v>15145.3</v>
+        <v>14811.9666666666</v>
       </c>
       <c r="L17" s="171" t="n">
         <f aca="false">L15+L16</f>
-        <v>10797.3</v>
+        <v>10463.9666666666</v>
       </c>
       <c r="M17" s="171" t="n">
         <f aca="false">M15+M16</f>
-        <v>17283.05</v>
+        <v>16949.7166666666</v>
       </c>
       <c r="N17" s="171" t="n">
         <f aca="false">N15+N16</f>
-        <v>16479.8</v>
+        <v>16146.4666666666</v>
       </c>
       <c r="O17" s="171" t="n">
         <f aca="false">O15+O16</f>
-        <v>10408.6333333333</v>
+        <v>10075.3</v>
       </c>
       <c r="P17" s="159"/>
     </row>
@@ -30022,55 +30047,55 @@
       </c>
       <c r="C30" s="171" t="n">
         <f aca="false">SUM(D30:O30)</f>
-        <v>149665.316666667</v>
+        <v>153665.316666667</v>
       </c>
       <c r="D30" s="171" t="n">
         <f aca="false">IF(C5&gt;0,IF(D5&gt;0,D13,C13/C21),0)</f>
-        <v>12012.7833333333</v>
+        <v>12346.1166666667</v>
       </c>
       <c r="E30" s="171" t="n">
         <f aca="false">IF(C5&gt;0,IF(E5&gt;0,E13,C13/C21),0)</f>
-        <v>11323.5333333333</v>
+        <v>11656.8666666667</v>
       </c>
       <c r="F30" s="171" t="n">
         <f aca="false">IF(C5&gt;0,IF(F5&gt;0,F13,C13/C21),0)</f>
-        <v>13592.8666666667</v>
+        <v>13926.2</v>
       </c>
       <c r="G30" s="171" t="n">
         <f aca="false">IF(C5&gt;0,IF(G5&gt;0,G13,C13/C21),0)</f>
-        <v>13829.7833333333</v>
+        <v>14163.1166666667</v>
       </c>
       <c r="H30" s="171" t="n">
         <f aca="false">IF(C5&gt;0,IF(H5&gt;0,H13,C13/C21),0)</f>
-        <v>11766.1166666667</v>
+        <v>12099.45</v>
       </c>
       <c r="I30" s="171" t="n">
         <f aca="false">IF(C5&gt;0,IF(I5&gt;0,I13,C13/C21),0)</f>
-        <v>13242.8666666667</v>
+        <v>13576.2</v>
       </c>
       <c r="J30" s="171" t="n">
         <f aca="false">IF(C5&gt;0,IF(J5&gt;0,J13,C13/C21),0)</f>
-        <v>13692.2833333333</v>
+        <v>14025.6166666667</v>
       </c>
       <c r="K30" s="171" t="n">
         <f aca="false">IF(C5&gt;0,IF(K5&gt;0,K13,C13/C21),0)</f>
-        <v>10880.5333333333</v>
+        <v>11213.8666666667</v>
       </c>
       <c r="L30" s="171" t="n">
         <f aca="false">IF(C5&gt;0,IF(L5&gt;0,L13,C13/C21),0)</f>
-        <v>15898.5333333333</v>
+        <v>16231.8666666667</v>
       </c>
       <c r="M30" s="171" t="n">
         <f aca="false">IF(C5&gt;0,IF(M5&gt;0,M13,C13/C21),0)</f>
-        <v>11392.7833333333</v>
+        <v>11726.1166666667</v>
       </c>
       <c r="N30" s="171" t="n">
         <f aca="false">IF(C5&gt;0,IF(N5&gt;0,N13,C13/C21),0)</f>
-        <v>11066.0333333333</v>
+        <v>11399.3666666667</v>
       </c>
       <c r="O30" s="171" t="n">
         <f aca="false">IF(C5&gt;0,IF(O5&gt;0,O13,C13/C21),0)</f>
-        <v>10967.2</v>
+        <v>11300.5333333333</v>
       </c>
       <c r="P30" s="159"/>
     </row>
@@ -30099,55 +30124,55 @@
       </c>
       <c r="C32" s="171" t="n">
         <f aca="false">SUM(D32:O32)</f>
-        <v>171481.35</v>
+        <v>167481.35</v>
       </c>
       <c r="D32" s="171" t="n">
         <f aca="false">D28-D30</f>
-        <v>15083.05</v>
+        <v>14749.7166666666</v>
       </c>
       <c r="E32" s="171" t="n">
         <f aca="false">E28-E30</f>
-        <v>15102.3</v>
+        <v>14768.9666666666</v>
       </c>
       <c r="F32" s="171" t="n">
         <f aca="false">F28-F30</f>
-        <v>11036.3</v>
+        <v>10702.9666666666</v>
       </c>
       <c r="G32" s="171" t="n">
         <f aca="false">G28-G30</f>
-        <v>13096.05</v>
+        <v>12762.7166666666</v>
       </c>
       <c r="H32" s="171" t="n">
         <f aca="false">H28-H30</f>
-        <v>17563.05</v>
+        <v>17229.7166666666</v>
       </c>
       <c r="I32" s="171" t="n">
         <f aca="false">I28-I30</f>
-        <v>14182.9666666666</v>
+        <v>13849.6333333333</v>
       </c>
       <c r="J32" s="171" t="n">
         <f aca="false">J28-J30</f>
-        <v>15303.55</v>
+        <v>14970.2166666666</v>
       </c>
       <c r="K32" s="171" t="n">
         <f aca="false">K28-K30</f>
-        <v>15145.3</v>
+        <v>14811.9666666666</v>
       </c>
       <c r="L32" s="171" t="n">
         <f aca="false">L28-L30</f>
-        <v>10797.3</v>
+        <v>10463.9666666666</v>
       </c>
       <c r="M32" s="171" t="n">
         <f aca="false">M28-M30</f>
-        <v>17283.05</v>
+        <v>16949.7166666666</v>
       </c>
       <c r="N32" s="171" t="n">
         <f aca="false">N28-N30</f>
-        <v>16479.8</v>
+        <v>16146.4666666666</v>
       </c>
       <c r="O32" s="171" t="n">
         <f aca="false">O28-O30</f>
-        <v>10408.6333333333</v>
+        <v>10075.3</v>
       </c>
       <c r="P32" s="159"/>
     </row>
@@ -30217,55 +30242,55 @@
       </c>
       <c r="C34" s="171" t="n">
         <f aca="false">SUM(D34:O34)</f>
-        <v>171481.35</v>
+        <v>167481.35</v>
       </c>
       <c r="D34" s="171" t="n">
         <f aca="false">D32+D33</f>
-        <v>15083.05</v>
+        <v>14749.7166666666</v>
       </c>
       <c r="E34" s="171" t="n">
         <f aca="false">E32+E33</f>
-        <v>15102.3</v>
+        <v>14768.9666666666</v>
       </c>
       <c r="F34" s="171" t="n">
         <f aca="false">F32+F33</f>
-        <v>11036.3</v>
+        <v>10702.9666666666</v>
       </c>
       <c r="G34" s="171" t="n">
         <f aca="false">G32+G33</f>
-        <v>13096.05</v>
+        <v>12762.7166666666</v>
       </c>
       <c r="H34" s="171" t="n">
         <f aca="false">H32+H33</f>
-        <v>17563.05</v>
+        <v>17229.7166666666</v>
       </c>
       <c r="I34" s="171" t="n">
         <f aca="false">I32+I33</f>
-        <v>14182.9666666666</v>
+        <v>13849.6333333333</v>
       </c>
       <c r="J34" s="171" t="n">
         <f aca="false">J32+J33</f>
-        <v>15303.55</v>
+        <v>14970.2166666666</v>
       </c>
       <c r="K34" s="171" t="n">
         <f aca="false">K32+K33</f>
-        <v>15145.3</v>
+        <v>14811.9666666666</v>
       </c>
       <c r="L34" s="171" t="n">
         <f aca="false">L32+L33</f>
-        <v>10797.3</v>
+        <v>10463.9666666666</v>
       </c>
       <c r="M34" s="171" t="n">
         <f aca="false">M32+M33</f>
-        <v>17283.05</v>
+        <v>16949.7166666666</v>
       </c>
       <c r="N34" s="171" t="n">
         <f aca="false">N32+N33</f>
-        <v>16479.8</v>
+        <v>16146.4666666666</v>
       </c>
       <c r="O34" s="171" t="n">
         <f aca="false">O32+O33</f>
-        <v>10408.6333333333</v>
+        <v>10075.3</v>
       </c>
       <c r="P34" s="159"/>
     </row>
@@ -30314,7 +30339,7 @@
       </c>
       <c r="C37" s="340" t="n">
         <f aca="false">'Profit &amp; Loss Account'!B33+'Profit &amp; Loss Account'!B34</f>
-        <v>13912</v>
+        <v>17912</v>
       </c>
       <c r="D37" s="159"/>
       <c r="E37" s="159"/>
@@ -30336,8 +30361,8 @@
         <v>390</v>
       </c>
       <c r="C38" s="340" t="n">
-        <f aca="false">[1]Schedule!$Q$1+[1]Schedule!$R$1+[1]Schedule!$Y$1-[1]Schedule!$Z$1</f>
-        <v>64000</v>
+        <f aca="false">[1]Schedule!$Q$1+[1]Schedule!$R$1+[1]Schedule!$AC$1+[1]Schedule!$Y$1-[1]Schedule!$Z$1</f>
+        <v>64540</v>
       </c>
       <c r="D38" s="159"/>
       <c r="E38" s="159"/>
@@ -30360,7 +30385,7 @@
       </c>
       <c r="C39" s="340" t="n">
         <f aca="false">C34+C37-C38</f>
-        <v>121393.35</v>
+        <v>120853.35</v>
       </c>
       <c r="D39" s="159"/>
       <c r="E39" s="159"/>
@@ -30383,7 +30408,7 @@
       </c>
       <c r="C40" s="340" t="n">
         <f aca="false">IF(C39&lt;=0,0,MAX(0,Admin!N$4-MAX(0,C39-Admin!N$5)/2))</f>
-        <v>1873.3250000002</v>
+        <v>2143.32500000022</v>
       </c>
       <c r="D40" s="159"/>
       <c r="E40" s="159"/>
@@ -30406,7 +30431,7 @@
       </c>
       <c r="C41" s="340" t="n">
         <f aca="false">IF((C39&gt;C40),(C39-C40),0)</f>
-        <v>119520.024999999</v>
+        <v>118710.024999999</v>
       </c>
       <c r="D41" s="159"/>
       <c r="E41" s="159"/>
@@ -30452,7 +30477,7 @@
       </c>
       <c r="C43" s="340" t="n">
         <f aca="false">IF(C41&gt;Admin!M$11,(MIN(C41,Admin!N$13)-Admin!M$11)*Admin!N$7,0)</f>
-        <v>32728.0099999998</v>
+        <v>32404.0099999997</v>
       </c>
       <c r="D43" s="159"/>
       <c r="E43" s="159"/>
@@ -30498,7 +30523,7 @@
       </c>
       <c r="C45" s="340" t="n">
         <f aca="false">IF(C39&gt;Admin!N$20,IF(C39&lt;Admin!N$23,(C39-Admin!N$20)*Admin!L$20,(Admin!N$23-Admin!N$20)*Admin!L$20),0)+IF(C39&gt;Admin!N$23,(C39-Admin!N$23)*Admin!L$23,0)</f>
-        <v>3684.46699999999</v>
+        <v>3673.66699999999</v>
       </c>
       <c r="D45" s="159"/>
       <c r="E45" s="159"/>
@@ -30521,7 +30546,7 @@
       </c>
       <c r="C46" s="342" t="n">
         <f aca="false">C42+C43+C44+C45</f>
-        <v>43952.4769999998</v>
+        <v>43617.6769999997</v>
       </c>
       <c r="D46" s="159"/>
       <c r="E46" s="159"/>

</xml_diff>

<commit_message>
SET-12: regenerate the SE packages, reports, example and parity fixture
The seven committed SE packages, the three Apr27 reconciliation reports,
examples/se-latest, the parity fixtures and the provenance stamp follow
the box 73 and box 77 formulas. On the recalculated advanced package box
73 reads 124,009.48 (was 123,919.48), box 76 126,092.81 (was 126,002.81),
income tax 42,944.76 (was 42,904.26), box 77 0 (was -90). The SE report
scorecard is 7,956 passed, the box 73 warning gone.

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Model: claude-opus-5
Claude-Session: https://claude.ai/code/session_01L9gReHshKw4uCy73kSr1AZ
</commit_message>
<xml_diff>
--- a/examples/se-latest/Financialaccounts.xlsx
+++ b/examples/se-latest/Financialaccounts.xlsx
@@ -20149,8 +20149,8 @@
         <v>33</v>
       </c>
       <c r="O194" s="98" t="n">
-        <f aca="false">O174</f>
-        <v>123919.475166666</v>
+        <f aca="false">MAX(0,O174-O179+N(D197)+D210+N(O190))</f>
+        <v>124009.475166666</v>
       </c>
       <c r="P194" s="98"/>
       <c r="Q194" s="98"/>
@@ -20627,7 +20627,7 @@
       </c>
       <c r="O210" s="98" t="n">
         <f aca="false">O194-O199+O204</f>
-        <v>126002.8085</v>
+        <v>126092.8085</v>
       </c>
       <c r="P210" s="98"/>
       <c r="Q210" s="98"/>
@@ -20872,8 +20872,8 @@
         <v>33</v>
       </c>
       <c r="D219" s="98" t="n">
-        <f aca="false">O179-N(D197)-D210-N(O190)</f>
-        <v>-90</v>
+        <f aca="false">MAX(0,O179-O174-N(D197)-D210-N(O190))</f>
+        <v>0</v>
       </c>
       <c r="E219" s="98"/>
       <c r="F219" s="98"/>
@@ -21051,7 +21051,7 @@
       </c>
       <c r="O224" s="98" t="n">
         <f aca="false">D219</f>
-        <v>-90</v>
+        <v>0</v>
       </c>
       <c r="P224" s="98"/>
       <c r="Q224" s="98"/>
@@ -30395,7 +30395,7 @@
       <c r="D5" s="222"/>
       <c r="E5" s="223" t="n">
         <f aca="false">'SE Full'!O210</f>
-        <v>126002.8085</v>
+        <v>126092.8085</v>
       </c>
       <c r="F5" s="214"/>
       <c r="G5" s="218"/>
@@ -30428,7 +30428,7 @@
       <c r="D7" s="222"/>
       <c r="E7" s="223" t="n">
         <f aca="false">IF((E5&gt;E6),(E5-E6),0)</f>
-        <v>126002.8085</v>
+        <v>126092.8085</v>
       </c>
       <c r="F7" s="214"/>
       <c r="G7" s="218"/>
@@ -30492,7 +30492,7 @@
       </c>
       <c r="E10" s="213" t="n">
         <f aca="false">IF(E7&gt;C10,(E7-C10)*D10,0)</f>
-        <v>388.263824999816</v>
+        <v>428.763824999816</v>
       </c>
       <c r="F10" s="214"/>
       <c r="G10" s="218"/>
@@ -30507,7 +30507,7 @@
       <c r="D11" s="230"/>
       <c r="E11" s="231" t="n">
         <f aca="false">SUM(E8:E10)</f>
-        <v>42904.2638249998</v>
+        <v>42944.7638249998</v>
       </c>
       <c r="F11" s="232"/>
       <c r="G11" s="233"/>
@@ -30583,7 +30583,7 @@
       </c>
       <c r="E16" s="240" t="n">
         <f aca="false">IF((E5&gt;Admin!N$23),((E5-Admin!N$23)*D16),0)</f>
-        <v>1514.65616999999</v>
+        <v>1516.45616999999</v>
       </c>
       <c r="F16" s="214"/>
       <c r="G16" s="233"/>
@@ -30608,7 +30608,7 @@
       <c r="D18" s="237"/>
       <c r="E18" s="231" t="n">
         <f aca="false">SUM(E11:E17)</f>
-        <v>46680.9199949998</v>
+        <v>46723.2199949998</v>
       </c>
       <c r="F18" s="214"/>
       <c r="G18" s="218"/>
@@ -31190,7 +31190,7 @@
       </c>
       <c r="E25" s="240" t="n">
         <f aca="false">E18</f>
-        <v>46680.9199949998</v>
+        <v>46723.2199949998</v>
       </c>
       <c r="F25" s="214"/>
       <c r="G25" s="218"/>
@@ -31207,7 +31207,7 @@
       </c>
       <c r="E26" s="223" t="n">
         <f aca="false">E25/2</f>
-        <v>23340.4599974999</v>
+        <v>23361.6099974999</v>
       </c>
       <c r="F26" s="214"/>
       <c r="G26" s="218"/>
@@ -31224,7 +31224,7 @@
       </c>
       <c r="E27" s="223" t="n">
         <f aca="false">E25/2</f>
-        <v>23340.4599974999</v>
+        <v>23361.6099974999</v>
       </c>
       <c r="F27" s="214"/>
       <c r="G27" s="218"/>

</xml_diff>

<commit_message>
SET-10: regenerate the SE packages, reports, example and parity fixture
The seven committed SE packages (Financialaccounts.xlsx and
Fixedassets.xlsx) carry the AH/AI split and the per-pool O144/D85
formula. On the recalculated 2026-27 advanced package, at that year's
14% main rate: the van's main pool balance is 24,000 (3,360 allowance,
20,640 written down) and the estate car's special rate pool 9,000 (540
allowance, 8,460 written down), both over £1,000, so O144 stays 0; the
hatchback's single asset pool figures (784, 0, 7,216) do not move. The
Apr27 advanced report, examples/se-latest, examples/parity/se and the
reconciliation page follow. The provenance stamp's reconciledCommit
records this branch's SET-10 code commit.

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Model: claude-sonnet-5
Claude-Session: coordinator dispatch, SET-10
</commit_message>
<xml_diff>
--- a/examples/se-latest/Financialaccounts.xlsx
+++ b/examples/se-latest/Financialaccounts.xlsx
@@ -4396,9 +4396,6 @@
           <cell r="R1">
             <v>4144</v>
           </cell>
-          <cell r="S1">
-            <v>36316</v>
-          </cell>
         </row>
         <row r="1">
           <cell r="V1">
@@ -4429,8 +4426,13 @@
           <cell r="AF1">
             <v>0</v>
           </cell>
-          <cell r="AG1">
-            <v>7216</v>
+        </row>
+        <row r="1">
+          <cell r="AH1">
+            <v>20640</v>
+          </cell>
+          <cell r="AI1">
+            <v>8460</v>
           </cell>
         </row>
       </sheetData>
@@ -12498,7 +12500,7 @@
         <v>33</v>
       </c>
       <c r="D85" s="98" t="n">
-        <f aca="false">IF(([1]Schedule!$R$1+[1]Schedule!$S$1-[1]Schedule!$AE$1-[1]Schedule!$AF$1-[1]Schedule!$AG$1)&lt;1000,[1]Schedule!$S$1-[1]Schedule!$AG$1,0)</f>
+        <f aca="false">IF(([1]Schedule!$R$1-[1]Schedule!$AE$1+[1]Schedule!$AH$1)&lt;1000,[1]Schedule!$AH$1,0)+IF(([1]Schedule!$AC$1-[1]Schedule!$AF$1+[1]Schedule!$AI$1)&lt;1000,[1]Schedule!$AI$1,0)</f>
         <v>0</v>
       </c>
       <c r="E85" s="98"/>
@@ -18641,7 +18643,7 @@
         <v>33</v>
       </c>
       <c r="O144" s="98" t="n">
-        <f aca="false">IF(([1]Schedule!$R$1+[1]Schedule!$S$1-[1]Schedule!$AE$1-[1]Schedule!$AF$1-[1]Schedule!$AG$1)&lt;1000,[1]Schedule!$S$1-[1]Schedule!$AG$1,0)</f>
+        <f aca="false">IF(([1]Schedule!$R$1-[1]Schedule!$AE$1+[1]Schedule!$AH$1)&lt;1000,[1]Schedule!$AH$1,0)+IF(([1]Schedule!$AC$1-[1]Schedule!$AF$1+[1]Schedule!$AI$1)&lt;1000,[1]Schedule!$AI$1,0)</f>
         <v>0</v>
       </c>
       <c r="P144" s="98"/>

</xml_diff>

<commit_message>
SET-9: regenerate the SE packages, reports, example and parity fixture
node app/bin/generate.js --package se, node app/bin/reconcile.js
--package se --scenario advanced --year-end 2027-04-05 (RECONCILES,
914/919 checks: box 53 = 1,800 exactly, box 53.1 = 1,024.66), node
diya-gl/scripts/parity-fixtures.mjs, node scripts/build-provenance-
data.mjs, node app/bin/build-reconciliation-pages.js --product se
--reports reports. examples/se-latest replaced with the freshly
populated 2026-27 Apr27 package, so the parity refresh reads a package
whose Schedule carries the new SBA block.

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Model: claude-sonnet-5
Claude-Session: https://claude.ai/code/session_01QJXZHSm9xjGESTWNSpV2bs
</commit_message>
<xml_diff>
--- a/examples/se-latest/Financialaccounts.xlsx
+++ b/examples/se-latest/Financialaccounts.xlsx
@@ -208,7 +208,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="800" uniqueCount="440">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="805" uniqueCount="443">
   <si>
     <r>
       <rPr>
@@ -1216,16 +1216,19 @@
     <t xml:space="preserve">Zero-emission goods vehicle allowance</t>
   </si>
   <si>
+    <t xml:space="preserve">Zero-emission car allowance</t>
+  </si>
+  <si>
     <t xml:space="preserve">Total capital allowances (total of boxes 49 to 56)</t>
   </si>
   <si>
-    <t xml:space="preserve">Zero-emission car allowance</t>
+    <t xml:space="preserve">The Structures and Buildings Allowance</t>
   </si>
   <si>
     <t xml:space="preserve">Balancing charge on sales of assets or on the cessation of</t>
   </si>
   <si>
-    <t xml:space="preserve">The Structures and Buildings Allowance</t>
+    <t xml:space="preserve">Freeport and Investment Zones Structures and Buildings Allowance</t>
   </si>
   <si>
     <t xml:space="preserve">business use (including where Business Premises Renovation</t>
@@ -2004,6 +2007,9 @@
     <t xml:space="preserve">Additional rate applicable above the higher rate limit</t>
   </si>
   <si>
+    <t xml:space="preserve">Structures and buildings allowance</t>
+  </si>
+  <si>
     <t xml:space="preserve">Taxable Bands Allowances</t>
   </si>
   <si>
@@ -2014,6 +2020,9 @@
   </si>
   <si>
     <t xml:space="preserve"> Tax Band </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Freeport and Investment Zone SBA</t>
   </si>
   <si>
     <t xml:space="preserve">Depreciation Rates Applied</t>
@@ -4435,6 +4444,16 @@
             <v>8460</v>
           </cell>
         </row>
+        <row r="120">
+          <cell r="K120">
+            <v>1800</v>
+          </cell>
+        </row>
+        <row r="121">
+          <cell r="K121">
+            <v>1024.65753424658</v>
+          </cell>
+        </row>
       </sheetData>
       <sheetData sheetId="1"/>
       <sheetData sheetId="2"/>
@@ -8760,7 +8779,7 @@
     <row r="1" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="63"/>
       <c r="B1" s="344" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C1" s="63"/>
       <c r="D1" s="345"/>
@@ -8783,7 +8802,7 @@
       </c>
       <c r="C2" s="63"/>
       <c r="D2" s="348" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="E2" s="348"/>
       <c r="F2" s="348"/>
@@ -8794,7 +8813,7 @@
       <c r="H2" s="63"/>
       <c r="I2" s="63"/>
       <c r="J2" s="350" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="K2" s="350"/>
       <c r="L2" s="348" t="str">
@@ -8840,7 +8859,7 @@
       </c>
       <c r="H4" s="63"/>
       <c r="I4" s="354" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="J4" s="354"/>
       <c r="K4" s="354"/>
@@ -8860,7 +8879,7 @@
       </c>
       <c r="C5" s="63"/>
       <c r="D5" s="354" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E5" s="354"/>
       <c r="F5" s="354"/>
@@ -8869,7 +8888,7 @@
       </c>
       <c r="H5" s="63"/>
       <c r="I5" s="354" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="J5" s="354"/>
       <c r="K5" s="354"/>
@@ -8889,7 +8908,7 @@
       </c>
       <c r="C6" s="63"/>
       <c r="D6" s="63" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="E6" s="63"/>
       <c r="F6" s="63"/>
@@ -8898,7 +8917,7 @@
       </c>
       <c r="H6" s="63"/>
       <c r="I6" s="354" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="J6" s="354"/>
       <c r="K6" s="354"/>
@@ -8908,7 +8927,7 @@
         <v>0.2</v>
       </c>
       <c r="O6" s="351" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8918,14 +8937,14 @@
       </c>
       <c r="C7" s="63"/>
       <c r="D7" s="354" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="E7" s="354"/>
       <c r="F7" s="354"/>
       <c r="G7" s="351"/>
       <c r="H7" s="63"/>
       <c r="I7" s="354" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="J7" s="354"/>
       <c r="K7" s="354"/>
@@ -8935,7 +8954,7 @@
         <v>0.4</v>
       </c>
       <c r="O7" s="351" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8950,7 +8969,7 @@
       <c r="G8" s="357"/>
       <c r="H8" s="63"/>
       <c r="I8" s="354" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="J8" s="354"/>
       <c r="K8" s="354"/>
@@ -8960,7 +8979,7 @@
         <v>0.45</v>
       </c>
       <c r="O8" s="351" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8969,24 +8988,28 @@
         <v>46265</v>
       </c>
       <c r="C9" s="63"/>
-      <c r="D9" s="63"/>
+      <c r="D9" s="63" t="s">
+        <v>412</v>
+      </c>
       <c r="E9" s="351"/>
       <c r="F9" s="63"/>
-      <c r="G9" s="351"/>
+      <c r="G9" s="355" t="n">
+        <v>0.03</v>
+      </c>
       <c r="H9" s="63"/>
       <c r="I9" s="354" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="J9" s="354"/>
       <c r="K9" s="354"/>
       <c r="L9" s="358" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="M9" s="358" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="N9" s="359" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="O9" s="351"/>
     </row>
@@ -8996,10 +9019,14 @@
         <v>46295</v>
       </c>
       <c r="C10" s="63"/>
-      <c r="D10" s="63"/>
+      <c r="D10" s="63" t="s">
+        <v>417</v>
+      </c>
       <c r="E10" s="351"/>
       <c r="F10" s="63"/>
-      <c r="G10" s="351"/>
+      <c r="G10" s="355" t="n">
+        <v>0.1</v>
+      </c>
       <c r="H10" s="63"/>
       <c r="I10" s="63"/>
       <c r="J10" s="63"/>
@@ -9016,16 +9043,16 @@
       </c>
       <c r="C11" s="63"/>
       <c r="D11" s="348" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="E11" s="348"/>
       <c r="F11" s="348"/>
       <c r="G11" s="351" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="H11" s="63"/>
       <c r="I11" s="63" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="J11" s="63"/>
       <c r="K11" s="360" t="n">
@@ -9055,7 +9082,7 @@
       <c r="G12" s="351"/>
       <c r="H12" s="63"/>
       <c r="I12" s="63" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="J12" s="63"/>
       <c r="K12" s="360" t="n">
@@ -9077,7 +9104,7 @@
       </c>
       <c r="C13" s="63"/>
       <c r="D13" s="354" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="E13" s="354"/>
       <c r="F13" s="354"/>
@@ -9086,7 +9113,7 @@
       </c>
       <c r="H13" s="63"/>
       <c r="I13" s="63" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="J13" s="63"/>
       <c r="K13" s="360" t="n">
@@ -9108,7 +9135,7 @@
       </c>
       <c r="C14" s="63"/>
       <c r="D14" s="354" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="E14" s="354"/>
       <c r="F14" s="354"/>
@@ -9117,7 +9144,7 @@
       </c>
       <c r="H14" s="63"/>
       <c r="I14" s="348" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="J14" s="348"/>
       <c r="K14" s="348"/>
@@ -9136,7 +9163,7 @@
       </c>
       <c r="C15" s="63"/>
       <c r="D15" s="354" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="E15" s="354"/>
       <c r="F15" s="354"/>
@@ -9159,7 +9186,7 @@
       </c>
       <c r="C16" s="63"/>
       <c r="D16" s="354" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="E16" s="354"/>
       <c r="F16" s="354"/>
@@ -9168,7 +9195,7 @@
       </c>
       <c r="H16" s="63"/>
       <c r="I16" s="354" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="J16" s="354"/>
       <c r="K16" s="354"/>
@@ -9176,7 +9203,7 @@
         <v>3.65</v>
       </c>
       <c r="M16" s="63" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="N16" s="357" t="n">
         <v>7105</v>
@@ -9192,7 +9219,7 @@
       </c>
       <c r="C17" s="63"/>
       <c r="D17" s="354" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="E17" s="354"/>
       <c r="F17" s="354"/>
@@ -9234,24 +9261,24 @@
       </c>
       <c r="C19" s="63"/>
       <c r="D19" s="348" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="E19" s="348"/>
       <c r="F19" s="351" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="G19" s="351" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="H19" s="63"/>
       <c r="I19" s="363" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="J19" s="363"/>
       <c r="K19" s="363"/>
       <c r="L19" s="63"/>
       <c r="M19" s="364" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="N19" s="63"/>
       <c r="O19" s="63"/>
@@ -9288,7 +9315,7 @@
       </c>
       <c r="C21" s="63"/>
       <c r="D21" s="354" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="E21" s="354"/>
       <c r="F21" s="357" t="n">
@@ -9313,7 +9340,7 @@
       </c>
       <c r="C22" s="63"/>
       <c r="D22" s="63" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="E22" s="63"/>
       <c r="F22" s="357" t="n">
@@ -9324,13 +9351,13 @@
       </c>
       <c r="H22" s="63"/>
       <c r="I22" s="363" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="J22" s="363"/>
       <c r="K22" s="363"/>
       <c r="L22" s="63"/>
       <c r="M22" s="364" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="N22" s="63"/>
       <c r="O22" s="63"/>
@@ -9338,7 +9365,7 @@
     <row r="23" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="63"/>
       <c r="B23" s="353" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="C23" s="63"/>
       <c r="D23" s="63"/>
@@ -9363,11 +9390,11 @@
     <row r="24" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="63"/>
       <c r="B24" s="353" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="C24" s="63"/>
       <c r="D24" s="348" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="E24" s="348"/>
       <c r="F24" s="63"/>
@@ -9405,7 +9432,7 @@
       <c r="B26" s="367"/>
       <c r="C26" s="63"/>
       <c r="D26" s="354" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E26" s="354"/>
       <c r="F26" s="357" t="n">
@@ -9426,7 +9453,7 @@
       <c r="B27" s="367"/>
       <c r="C27" s="63"/>
       <c r="D27" s="63" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="E27" s="63"/>
       <c r="F27" s="355" t="n">
@@ -18822,16 +18849,24 @@
       <c r="V149" s="63"/>
       <c r="W149" s="82"/>
     </row>
-    <row r="150" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="150" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A150" s="79"/>
       <c r="B150" s="63"/>
-      <c r="C150" s="64"/>
-      <c r="D150" s="63"/>
-      <c r="E150" s="63"/>
-      <c r="F150" s="63"/>
-      <c r="G150" s="63"/>
-      <c r="H150" s="63"/>
-      <c r="I150" s="63"/>
+      <c r="C150" s="97" t="s">
+        <v>33</v>
+      </c>
+      <c r="D150" s="98"/>
+      <c r="E150" s="98"/>
+      <c r="F150" s="98"/>
+      <c r="G150" s="99" t="s">
+        <v>34</v>
+      </c>
+      <c r="H150" s="100" t="n">
+        <v>0</v>
+      </c>
+      <c r="I150" s="100" t="n">
+        <v>0</v>
+      </c>
       <c r="J150" s="63"/>
       <c r="K150" s="63"/>
       <c r="L150" s="63"/>
@@ -18848,9 +18883,13 @@
       <c r="W150" s="82"/>
     </row>
     <row r="151" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A151" s="106"/>
+      <c r="A151" s="75" t="n">
+        <v>52.1</v>
+      </c>
       <c r="B151" s="63"/>
-      <c r="C151" s="64"/>
+      <c r="C151" s="64" t="s">
+        <v>167</v>
+      </c>
       <c r="D151" s="64"/>
       <c r="E151" s="64"/>
       <c r="F151" s="64"/>
@@ -18864,7 +18903,7 @@
       </c>
       <c r="M151" s="63"/>
       <c r="N151" s="64" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="O151" s="63"/>
       <c r="P151" s="63"/>
@@ -18882,7 +18921,9 @@
       <c r="C152" s="97" t="s">
         <v>33</v>
       </c>
-      <c r="D152" s="98"/>
+      <c r="D152" s="98" t="n">
+        <v>2500</v>
+      </c>
       <c r="E152" s="98"/>
       <c r="F152" s="98"/>
       <c r="G152" s="99" t="s">
@@ -18936,11 +18977,11 @@
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="75" t="n">
-        <v>52.1</v>
+        <v>53</v>
       </c>
       <c r="B154" s="63"/>
       <c r="C154" s="64" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D154" s="64"/>
       <c r="E154" s="64"/>
@@ -18956,8 +18997,8 @@
         <v>33</v>
       </c>
       <c r="O154" s="98" t="n">
-        <f aca="false">D139+D144+D147+D152+D156+D160+O139+O144+O149</f>
-        <v>69624</v>
+        <f aca="false">D139+D144+D147+D150+D152+D156+D160+O139+O144+O149</f>
+        <v>70648.6575342466</v>
       </c>
       <c r="P154" s="98"/>
       <c r="Q154" s="98"/>
@@ -19006,7 +19047,8 @@
         <v>33</v>
       </c>
       <c r="D156" s="98" t="n">
-        <v>2500</v>
+        <f aca="false">[1]Schedule!$K$120</f>
+        <v>1800</v>
       </c>
       <c r="E156" s="98"/>
       <c r="F156" s="98"/>
@@ -19026,7 +19068,7 @@
       </c>
       <c r="M156" s="63"/>
       <c r="N156" s="64" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="O156" s="63"/>
       <c r="P156" s="63"/>
@@ -19040,11 +19082,11 @@
     </row>
     <row r="157" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="75" t="n">
-        <v>53</v>
+        <v>53.1</v>
       </c>
       <c r="B157" s="63"/>
       <c r="C157" s="64" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D157" s="64"/>
       <c r="E157" s="64"/>
@@ -19057,7 +19099,7 @@
       <c r="L157" s="63"/>
       <c r="M157" s="63"/>
       <c r="N157" s="64" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="O157" s="63"/>
       <c r="P157" s="63"/>
@@ -19084,7 +19126,7 @@
       <c r="L158" s="63"/>
       <c r="M158" s="63"/>
       <c r="N158" s="64" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="O158" s="63"/>
       <c r="P158" s="63"/>
@@ -19128,7 +19170,8 @@
         <v>33</v>
       </c>
       <c r="D160" s="98" t="n">
-        <v>1800</v>
+        <f aca="false">[1]Schedule!$K$121</f>
+        <v>1024.65753424658</v>
       </c>
       <c r="E160" s="98"/>
       <c r="F160" s="98"/>
@@ -19194,7 +19237,7 @@
     </row>
     <row r="162" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A162" s="103" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B162" s="103"/>
       <c r="C162" s="103"/>
@@ -19221,7 +19264,7 @@
     </row>
     <row r="163" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A163" s="104" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B163" s="104"/>
       <c r="C163" s="104"/>
@@ -19248,7 +19291,7 @@
     </row>
     <row r="164" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A164" s="104" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B164" s="104"/>
       <c r="C164" s="104"/>
@@ -19304,7 +19347,7 @@
       </c>
       <c r="B166" s="63"/>
       <c r="C166" s="64" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D166" s="64"/>
       <c r="E166" s="64"/>
@@ -19319,7 +19362,7 @@
       </c>
       <c r="M166" s="63"/>
       <c r="N166" s="64" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="O166" s="63"/>
       <c r="P166" s="63"/>
@@ -19346,7 +19389,7 @@
       <c r="L167" s="64"/>
       <c r="M167" s="63"/>
       <c r="N167" s="64" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="O167" s="110"/>
       <c r="P167" s="110"/>
@@ -19413,7 +19456,7 @@
       </c>
       <c r="O169" s="98" t="n">
         <f aca="false">O154+D179</f>
-        <v>69974</v>
+        <v>70998.6575342466</v>
       </c>
       <c r="P169" s="98"/>
       <c r="Q169" s="98"/>
@@ -19461,7 +19504,7 @@
       </c>
       <c r="B171" s="63"/>
       <c r="C171" s="64" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D171" s="64"/>
       <c r="E171" s="64"/>
@@ -19476,7 +19519,7 @@
       </c>
       <c r="M171" s="63"/>
       <c r="N171" s="64" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="O171" s="63"/>
       <c r="P171" s="63"/>
@@ -19492,7 +19535,7 @@
       <c r="A172" s="106"/>
       <c r="B172" s="63"/>
       <c r="C172" s="64" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D172" s="64"/>
       <c r="E172" s="64"/>
@@ -19505,7 +19548,7 @@
       <c r="L172" s="64"/>
       <c r="M172" s="63"/>
       <c r="N172" s="64" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="O172" s="63"/>
       <c r="P172" s="63"/>
@@ -19572,7 +19615,7 @@
       </c>
       <c r="O174" s="98" t="n">
         <f aca="false">IF((D129+D174-O169)&gt;0,(D129+D174-O169),IF((-O129+D174-O169)&gt;0,(-O129+D174-O169),0))</f>
-        <v>123135.475166666</v>
+        <v>122110.81763242</v>
       </c>
       <c r="P174" s="98"/>
       <c r="Q174" s="98"/>
@@ -19620,7 +19663,7 @@
       </c>
       <c r="B176" s="63"/>
       <c r="C176" s="64" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D176" s="64"/>
       <c r="E176" s="64"/>
@@ -19635,7 +19678,7 @@
       </c>
       <c r="M176" s="63"/>
       <c r="N176" s="64" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="O176" s="63"/>
       <c r="P176" s="63"/>
@@ -19651,7 +19694,7 @@
       <c r="A177" s="79"/>
       <c r="B177" s="63"/>
       <c r="C177" s="64" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D177" s="63"/>
       <c r="E177" s="63"/>
@@ -19664,7 +19707,7 @@
       <c r="L177" s="63"/>
       <c r="M177" s="63"/>
       <c r="N177" s="64" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="O177" s="63"/>
       <c r="P177" s="63"/>
@@ -19774,7 +19817,7 @@
     </row>
     <row r="181" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A181" s="103" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B181" s="103"/>
       <c r="C181" s="103"/>
@@ -19801,7 +19844,7 @@
     </row>
     <row r="182" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A182" s="104" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B182" s="104"/>
       <c r="C182" s="104"/>
@@ -19828,7 +19871,7 @@
     </row>
     <row r="183" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A183" s="104" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B183" s="104"/>
       <c r="C183" s="104"/>
@@ -19855,7 +19898,7 @@
     </row>
     <row r="184" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A184" s="133" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B184" s="133"/>
       <c r="C184" s="133"/>
@@ -19909,7 +19952,7 @@
       <c r="A186" s="75"/>
       <c r="B186" s="63"/>
       <c r="C186" s="64" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D186" s="64"/>
       <c r="E186" s="64"/>
@@ -19924,7 +19967,7 @@
       </c>
       <c r="M186" s="63"/>
       <c r="N186" s="64" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="O186" s="63"/>
       <c r="P186" s="63"/>
@@ -19951,7 +19994,7 @@
       <c r="L187" s="64"/>
       <c r="M187" s="63"/>
       <c r="N187" s="80" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="O187" s="63"/>
       <c r="P187" s="63"/>
@@ -19978,7 +20021,7 @@
       <c r="L188" s="64"/>
       <c r="M188" s="63"/>
       <c r="N188" s="92" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="O188" s="63"/>
       <c r="P188" s="63"/>
@@ -20005,7 +20048,7 @@
       <c r="L189" s="64"/>
       <c r="M189" s="63"/>
       <c r="N189" s="92" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="O189" s="110"/>
       <c r="P189" s="110"/>
@@ -20035,7 +20078,7 @@
         <v>33</v>
       </c>
       <c r="O190" s="136" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="P190" s="137"/>
       <c r="Q190" s="137"/>
@@ -20083,7 +20126,7 @@
       </c>
       <c r="B192" s="63"/>
       <c r="C192" s="64" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D192" s="112"/>
       <c r="E192" s="112"/>
@@ -20098,7 +20141,7 @@
       </c>
       <c r="M192" s="63"/>
       <c r="N192" s="64" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="O192" s="63"/>
       <c r="P192" s="63"/>
@@ -20117,7 +20160,7 @@
       <c r="A193" s="79"/>
       <c r="B193" s="63"/>
       <c r="C193" s="64" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D193" s="64"/>
       <c r="E193" s="64"/>
@@ -20130,7 +20173,7 @@
       <c r="L193" s="64"/>
       <c r="M193" s="64"/>
       <c r="N193" s="80" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="O193" s="112"/>
       <c r="P193" s="112"/>
@@ -20146,7 +20189,7 @@
       <c r="A194" s="79"/>
       <c r="B194" s="63"/>
       <c r="C194" s="80" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D194" s="64"/>
       <c r="E194" s="64"/>
@@ -20163,7 +20206,7 @@
       </c>
       <c r="O194" s="98" t="n">
         <f aca="false">MAX(0,O174-O179+N(D197)+D210+N(O190))</f>
-        <v>123225.475166666</v>
+        <v>122200.81763242</v>
       </c>
       <c r="P194" s="98"/>
       <c r="Q194" s="98"/>
@@ -20222,7 +20265,7 @@
       </c>
       <c r="M196" s="63"/>
       <c r="N196" s="64" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="O196" s="63"/>
       <c r="P196" s="63"/>
@@ -20241,7 +20284,7 @@
         <v>33</v>
       </c>
       <c r="D197" s="136" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="E197" s="137"/>
       <c r="F197" s="137"/>
@@ -20259,7 +20302,7 @@
       <c r="L197" s="63"/>
       <c r="M197" s="63"/>
       <c r="N197" s="80" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="O197" s="63"/>
       <c r="P197" s="63"/>
@@ -20300,7 +20343,7 @@
       <c r="A199" s="75"/>
       <c r="B199" s="63"/>
       <c r="C199" s="64" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D199" s="63"/>
       <c r="E199" s="63"/>
@@ -20376,7 +20419,7 @@
       </c>
       <c r="M201" s="63"/>
       <c r="N201" s="64" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="O201" s="63"/>
       <c r="P201" s="63"/>
@@ -20403,7 +20446,7 @@
       <c r="L202" s="63"/>
       <c r="M202" s="63"/>
       <c r="N202" s="64" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="O202" s="63"/>
       <c r="P202" s="63"/>
@@ -20545,7 +20588,7 @@
       <c r="L207" s="63"/>
       <c r="M207" s="63"/>
       <c r="N207" s="64" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="O207" s="63"/>
       <c r="P207" s="63"/>
@@ -20563,7 +20606,7 @@
       </c>
       <c r="B208" s="63"/>
       <c r="C208" s="64" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D208" s="64"/>
       <c r="E208" s="64"/>
@@ -20640,7 +20683,7 @@
       </c>
       <c r="O210" s="98" t="n">
         <f aca="false">O194-O199+O204</f>
-        <v>125308.8085</v>
+        <v>124284.150965753</v>
       </c>
       <c r="P210" s="98"/>
       <c r="Q210" s="98"/>
@@ -20684,7 +20727,7 @@
     </row>
     <row r="212" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A212" s="111" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B212" s="111"/>
       <c r="C212" s="111"/>
@@ -20711,7 +20754,7 @@
     </row>
     <row r="213" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A213" s="104" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B213" s="104"/>
       <c r="C213" s="104"/>
@@ -20738,7 +20781,7 @@
     </row>
     <row r="214" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A214" s="104" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B214" s="104"/>
       <c r="C214" s="104"/>
@@ -20794,7 +20837,7 @@
       </c>
       <c r="B216" s="63"/>
       <c r="C216" s="64" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D216" s="64"/>
       <c r="E216" s="64"/>
@@ -20803,7 +20846,7 @@
         <v>2026-27</v>
       </c>
       <c r="G216" s="64" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="H216" s="64"/>
       <c r="I216" s="64"/>
@@ -20814,7 +20857,7 @@
       </c>
       <c r="M216" s="63"/>
       <c r="N216" s="64" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="O216" s="63"/>
       <c r="P216" s="63"/>
@@ -20953,7 +20996,7 @@
       </c>
       <c r="B221" s="63"/>
       <c r="C221" s="64" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D221" s="64"/>
       <c r="E221" s="64"/>
@@ -21108,7 +21151,7 @@
     </row>
     <row r="226" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A226" s="147" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B226" s="147"/>
       <c r="C226" s="147"/>
@@ -21164,7 +21207,7 @@
       </c>
       <c r="B228" s="63"/>
       <c r="C228" s="64" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D228" s="64"/>
       <c r="E228" s="64"/>
@@ -21179,7 +21222,7 @@
       </c>
       <c r="M228" s="63"/>
       <c r="N228" s="64" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="O228" s="63"/>
       <c r="P228" s="63"/>
@@ -21195,7 +21238,7 @@
       <c r="A229" s="106"/>
       <c r="B229" s="63"/>
       <c r="C229" s="64" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D229" s="64"/>
       <c r="E229" s="64"/>
@@ -21314,7 +21357,7 @@
     </row>
     <row r="233" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A233" s="103" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B233" s="103"/>
       <c r="C233" s="103"/>
@@ -21341,7 +21384,7 @@
     </row>
     <row r="234" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A234" s="104" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B234" s="104"/>
       <c r="C234" s="104"/>
@@ -21368,7 +21411,7 @@
     </row>
     <row r="235" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A235" s="104" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B235" s="104"/>
       <c r="C235" s="104"/>
@@ -21422,7 +21465,7 @@
       <c r="A237" s="79"/>
       <c r="B237" s="63"/>
       <c r="C237" s="129" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D237" s="63"/>
       <c r="E237" s="63"/>
@@ -21435,7 +21478,7 @@
       <c r="L237" s="63"/>
       <c r="M237" s="63"/>
       <c r="N237" s="129" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="O237" s="63"/>
       <c r="P237" s="63"/>
@@ -21478,7 +21521,7 @@
       </c>
       <c r="B239" s="63"/>
       <c r="C239" s="64" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D239" s="64"/>
       <c r="E239" s="64"/>
@@ -21493,7 +21536,7 @@
       </c>
       <c r="M239" s="63"/>
       <c r="N239" s="64" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="O239" s="63"/>
       <c r="P239" s="63"/>
@@ -21602,7 +21645,7 @@
       </c>
       <c r="B243" s="63"/>
       <c r="C243" s="64" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D243" s="64"/>
       <c r="E243" s="64"/>
@@ -21617,7 +21660,7 @@
       </c>
       <c r="M243" s="63"/>
       <c r="N243" s="64" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="O243" s="63"/>
       <c r="P243" s="63"/>
@@ -21726,7 +21769,7 @@
       </c>
       <c r="B247" s="63"/>
       <c r="C247" s="64" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D247" s="64"/>
       <c r="E247" s="64"/>
@@ -21741,7 +21784,7 @@
       </c>
       <c r="M247" s="63"/>
       <c r="N247" s="64" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="O247" s="63"/>
       <c r="P247" s="63"/>
@@ -21850,7 +21893,7 @@
       </c>
       <c r="B251" s="63"/>
       <c r="C251" s="64" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D251" s="64"/>
       <c r="E251" s="64"/>
@@ -21863,7 +21906,7 @@
       <c r="L251" s="63"/>
       <c r="M251" s="63"/>
       <c r="N251" s="129" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="O251" s="112"/>
       <c r="P251" s="112"/>
@@ -21925,7 +21968,7 @@
       </c>
       <c r="M253" s="63"/>
       <c r="N253" s="64" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="O253" s="63"/>
       <c r="P253" s="63"/>
@@ -21968,7 +22011,7 @@
       </c>
       <c r="B255" s="63"/>
       <c r="C255" s="64" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D255" s="64"/>
       <c r="E255" s="64"/>
@@ -21984,7 +22027,7 @@
         <v>33</v>
       </c>
       <c r="O255" s="149" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="P255" s="98"/>
       <c r="Q255" s="98"/>
@@ -22049,7 +22092,7 @@
       <c r="L257" s="63"/>
       <c r="M257" s="63"/>
       <c r="N257" s="129" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="O257" s="63"/>
       <c r="P257" s="63"/>
@@ -22092,7 +22135,7 @@
       </c>
       <c r="B259" s="63"/>
       <c r="C259" s="64" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D259" s="64"/>
       <c r="E259" s="64"/>
@@ -22107,7 +22150,7 @@
       </c>
       <c r="M259" s="63"/>
       <c r="N259" s="64" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="O259" s="63"/>
       <c r="P259" s="63"/>
@@ -22170,7 +22213,7 @@
         <v>33</v>
       </c>
       <c r="O261" s="136" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="P261" s="98"/>
       <c r="Q261" s="98"/>
@@ -22218,7 +22261,7 @@
       </c>
       <c r="B263" s="63"/>
       <c r="C263" s="64" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D263" s="64"/>
       <c r="E263" s="64"/>
@@ -22233,7 +22276,7 @@
       </c>
       <c r="M263" s="63"/>
       <c r="N263" s="64" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="O263" s="63"/>
       <c r="P263" s="63"/>
@@ -22296,7 +22339,7 @@
         <v>33</v>
       </c>
       <c r="O265" s="136" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="P265" s="98"/>
       <c r="Q265" s="98"/>
@@ -22344,7 +22387,7 @@
       </c>
       <c r="B267" s="63"/>
       <c r="C267" s="64" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D267" s="64"/>
       <c r="E267" s="64"/>
@@ -22359,7 +22402,7 @@
       </c>
       <c r="M267" s="63"/>
       <c r="N267" s="64" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="O267" s="63"/>
       <c r="P267" s="63"/>
@@ -22479,7 +22522,7 @@
       </c>
       <c r="M271" s="63"/>
       <c r="N271" s="64" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="O271" s="63"/>
       <c r="P271" s="63"/>
@@ -22591,7 +22634,7 @@
       </c>
       <c r="M275" s="63"/>
       <c r="N275" s="64" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="O275" s="63"/>
       <c r="P275" s="63"/>
@@ -22646,7 +22689,7 @@
         <v>33</v>
       </c>
       <c r="O277" s="136" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="P277" s="98"/>
       <c r="Q277" s="98"/>
@@ -22690,7 +22733,7 @@
     </row>
     <row r="279" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A279" s="111" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B279" s="111"/>
       <c r="C279" s="111"/>
@@ -22717,7 +22760,7 @@
     </row>
     <row r="280" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A280" s="104" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B280" s="104"/>
       <c r="C280" s="104"/>
@@ -22732,7 +22775,7 @@
         <v>12570</v>
       </c>
       <c r="K280" s="104" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="L280" s="104"/>
       <c r="M280" s="104"/>
@@ -22749,7 +22792,7 @@
     </row>
     <row r="281" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A281" s="151" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B281" s="151"/>
       <c r="C281" s="151"/>
@@ -22805,7 +22848,7 @@
       </c>
       <c r="B283" s="63"/>
       <c r="C283" s="64" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D283" s="63"/>
       <c r="E283" s="63"/>
@@ -22820,7 +22863,7 @@
       </c>
       <c r="M283" s="63"/>
       <c r="N283" s="64" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="O283" s="63"/>
       <c r="P283" s="63"/>
@@ -22836,7 +22879,7 @@
       <c r="A284" s="79"/>
       <c r="B284" s="63"/>
       <c r="C284" s="64" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D284" s="63"/>
       <c r="E284" s="63"/>
@@ -22849,7 +22892,7 @@
       <c r="L284" s="63"/>
       <c r="M284" s="63"/>
       <c r="N284" s="90" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="O284" s="63"/>
       <c r="P284" s="63"/>
@@ -22950,7 +22993,7 @@
       </c>
       <c r="B288" s="63"/>
       <c r="C288" s="64" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D288" s="63"/>
       <c r="E288" s="63"/>
@@ -22977,7 +23020,7 @@
       <c r="A289" s="79"/>
       <c r="B289" s="63"/>
       <c r="C289" s="64" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D289" s="63"/>
       <c r="E289" s="63"/>
@@ -23102,7 +23145,7 @@
     </row>
     <row r="294" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A294" s="103" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B294" s="103"/>
       <c r="C294" s="103"/>
@@ -23158,7 +23201,7 @@
       </c>
       <c r="B296" s="63"/>
       <c r="C296" s="64" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D296" s="63"/>
       <c r="E296" s="63"/>
@@ -23882,7 +23925,7 @@
       <c r="W324" s="95"/>
     </row>
   </sheetData>
-  <mergeCells count="149">
+  <mergeCells count="150">
     <mergeCell ref="A1:F2"/>
     <mergeCell ref="G1:M2"/>
     <mergeCell ref="N1:W1"/>
@@ -23963,6 +24006,7 @@
     <mergeCell ref="H146:I146"/>
     <mergeCell ref="D147:F147"/>
     <mergeCell ref="O149:Q149"/>
+    <mergeCell ref="D150:F150"/>
     <mergeCell ref="D152:F152"/>
     <mergeCell ref="O154:Q154"/>
     <mergeCell ref="D156:F156"/>
@@ -24084,10 +24128,10 @@
     </row>
     <row r="2" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="160" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B2" s="161" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C2" s="162" t="n">
         <f aca="false">Admin!B5</f>
@@ -24204,7 +24248,7 @@
     </row>
     <row r="5" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="169" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B5" s="170" t="n">
         <f aca="false">SUM(C5:N5)</f>
@@ -24262,7 +24306,7 @@
     </row>
     <row r="6" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="169" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B6" s="170" t="n">
         <f aca="false">SUM(C6:N6)</f>
@@ -24320,7 +24364,7 @@
     </row>
     <row r="7" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="169" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B7" s="170" t="n">
         <f aca="false">SUM(C7:N7)</f>
@@ -24378,7 +24422,7 @@
     </row>
     <row r="8" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="169" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B8" s="170" t="n">
         <f aca="false">SUM(C8:N8)</f>
@@ -24436,7 +24480,7 @@
     </row>
     <row r="9" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="173" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B9" s="170" t="n">
         <f aca="false">SUM(B5:B8)</f>
@@ -24995,7 +25039,7 @@
     </row>
     <row r="11" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="169" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B11" s="170" t="n">
         <f aca="false">SUM(C11:N11)</f>
@@ -25312,7 +25356,7 @@
     </row>
     <row r="13" customFormat="false" ht="10.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="180" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B13" s="177"/>
       <c r="C13" s="177"/>
@@ -25573,7 +25617,7 @@
     </row>
     <row r="14" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="169" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B14" s="170" t="n">
         <f aca="false">SUM(C14:N14)</f>
@@ -25631,7 +25675,7 @@
     </row>
     <row r="15" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="169" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B15" s="170" t="n">
         <f aca="false">SUM(C15:N15)</f>
@@ -25689,7 +25733,7 @@
     </row>
     <row r="16" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="169" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B16" s="170" t="n">
         <f aca="false">SUM(C16:N16)</f>
@@ -25747,7 +25791,7 @@
     </row>
     <row r="17" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="173" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B17" s="170" t="n">
         <f aca="false">SUM(B14:B16)</f>
@@ -26306,7 +26350,7 @@
     </row>
     <row r="19" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="173" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B19" s="170" t="n">
         <f aca="false">B9+B11-B17</f>
@@ -26606,7 +26650,7 @@
     </row>
     <row r="20" customFormat="false" ht="10.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="180" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B20" s="177"/>
       <c r="C20" s="181"/>
@@ -26867,7 +26911,7 @@
     </row>
     <row r="21" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="169" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B21" s="170" t="n">
         <f aca="false">SUM(C21:N21)</f>
@@ -26925,7 +26969,7 @@
     </row>
     <row r="22" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="182" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B22" s="170" t="n">
         <f aca="false">SUM(C22:N22)</f>
@@ -26983,7 +27027,7 @@
     </row>
     <row r="23" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="182" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B23" s="170" t="n">
         <f aca="false">SUM(C23:N23)</f>
@@ -27041,7 +27085,7 @@
     </row>
     <row r="24" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="182" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B24" s="170" t="n">
         <f aca="false">SUM(C24:N24)</f>
@@ -27099,7 +27143,7 @@
     </row>
     <row r="25" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="182" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B25" s="170" t="n">
         <f aca="false">SUM(C25:N25)</f>
@@ -27157,7 +27201,7 @@
     </row>
     <row r="26" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="182" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B26" s="170" t="n">
         <f aca="false">SUM(C26:N26)</f>
@@ -27215,7 +27259,7 @@
     </row>
     <row r="27" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="182" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B27" s="170" t="n">
         <f aca="false">SUM(C27:N27)</f>
@@ -27273,7 +27317,7 @@
     </row>
     <row r="28" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="182" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B28" s="170" t="n">
         <f aca="false">SUM(C28:N28)</f>
@@ -27331,7 +27375,7 @@
     </row>
     <row r="29" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="182" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B29" s="170" t="n">
         <f aca="false">SUM(C29:N29)</f>
@@ -27389,7 +27433,7 @@
     </row>
     <row r="30" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="182" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B30" s="170" t="n">
         <f aca="false">SUM(C30:N30)</f>
@@ -27447,7 +27491,7 @@
     </row>
     <row r="31" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="182" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B31" s="170" t="n">
         <f aca="false">SUM(C31:N31)</f>
@@ -27505,7 +27549,7 @@
     </row>
     <row r="32" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="182" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B32" s="170" t="n">
         <f aca="false">SUM(C32:N32)</f>
@@ -27563,7 +27607,7 @@
     </row>
     <row r="33" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="169" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B33" s="170" t="n">
         <f aca="false">SUM(C33:N33)</f>
@@ -27621,7 +27665,7 @@
     </row>
     <row r="34" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="169" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B34" s="170" t="n">
         <f aca="false">SUM(C34:N34)</f>
@@ -27679,7 +27723,7 @@
     </row>
     <row r="35" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="173" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B35" s="170" t="n">
         <f aca="false">SUM(B21:B34)</f>
@@ -27754,7 +27798,7 @@
     </row>
     <row r="37" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="173" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B37" s="170" t="n">
         <f aca="false">B19-B35</f>
@@ -27812,7 +27856,7 @@
     </row>
     <row r="38" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="169" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B38" s="170" t="n">
         <f aca="false">SUM(C38:N38)</f>
@@ -27870,7 +27914,7 @@
     </row>
     <row r="39" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="173" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B39" s="170" t="n">
         <f aca="false">B37+B38</f>
@@ -27945,7 +27989,7 @@
     </row>
     <row r="41" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="187" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B41" s="156"/>
       <c r="C41" s="157"/>
@@ -27964,7 +28008,7 @@
     </row>
     <row r="42" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="182" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B42" s="177" t="n">
         <f aca="false">SUM(C42:N42)</f>
@@ -28022,7 +28066,7 @@
     </row>
     <row r="43" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="182" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B43" s="177" t="n">
         <f aca="false">SUM(C43:N43)</f>
@@ -28080,7 +28124,7 @@
     </row>
     <row r="44" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="182" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B44" s="177" t="n">
         <f aca="false">SUM(C44:N44)</f>
@@ -28138,7 +28182,7 @@
     </row>
     <row r="45" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="188" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B45" s="189" t="n">
         <f aca="false">SUM(C45:N45)</f>
@@ -28196,7 +28240,7 @@
     </row>
     <row r="46" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="182" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B46" s="177" t="n">
         <f aca="false">SUM(C46:N46)</f>
@@ -28271,7 +28315,7 @@
     </row>
     <row r="49" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="182" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B49" s="170" t="n">
         <f aca="false">SUM(C49:N49)</f>
@@ -28386,25 +28430,25 @@
     <row r="2" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="195"/>
       <c r="B2" s="197" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C2" s="197" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D2" s="197" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="E2" s="197" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F2" s="197" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="G2" s="197" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="H2" s="197" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="I2" s="195"/>
       <c r="J2" s="196"/>
@@ -28929,7 +28973,7 @@
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="195"/>
       <c r="B5" s="195" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C5" s="199" t="n">
         <f aca="false">SUM('Profit &amp; Loss Account'!C5:E7)</f>
@@ -28957,7 +29001,7 @@
     <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="195"/>
       <c r="B6" s="195" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C6" s="199" t="n">
         <f aca="false">SUM('Profit &amp; Loss Account'!C8:E8)+SUM('Profit &amp; Loss Account'!C11:E11)+SUM('Profit &amp; Loss Account'!C38:E38)</f>
@@ -28985,7 +29029,7 @@
     <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="195"/>
       <c r="B7" s="195" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C7" s="199" t="n">
         <f aca="false">SUM('Profit &amp; Loss Account'!C14:E14)+SUM('Profit &amp; Loss Account'!C16:E16)</f>
@@ -29283,7 +29327,7 @@
     <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="195"/>
       <c r="B10" s="202" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C10" s="195"/>
       <c r="D10" s="195"/>
@@ -29307,7 +29351,7 @@
     <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="195"/>
       <c r="B12" s="195" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C12" s="200" t="n">
         <f aca="false">SUM('Profit &amp; Loss Account'!C21:E21)</f>
@@ -29335,7 +29379,7 @@
     <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="195"/>
       <c r="B13" s="195" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C13" s="200" t="n">
         <f aca="false">SUM('Profit &amp; Loss Account'!C22:E22)</f>
@@ -29363,7 +29407,7 @@
     <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="195"/>
       <c r="B14" s="195" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C14" s="200" t="n">
         <f aca="false">SUM('Profit &amp; Loss Account'!C23:E23)</f>
@@ -29391,7 +29435,7 @@
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="195"/>
       <c r="B15" s="195" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C15" s="200" t="n">
         <f aca="false">SUM('Profit &amp; Loss Account'!C24:E24)</f>
@@ -29419,7 +29463,7 @@
     <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="195"/>
       <c r="B16" s="195" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C16" s="200" t="n">
         <f aca="false">SUM('Profit &amp; Loss Account'!C31:E31)</f>
@@ -29447,7 +29491,7 @@
     <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="195"/>
       <c r="B17" s="195" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C17" s="200" t="n">
         <f aca="false">SUM('Profit &amp; Loss Account'!C25:E26)</f>
@@ -29475,7 +29519,7 @@
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="195"/>
       <c r="B18" s="195" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C18" s="200" t="n">
         <f aca="false">SUM('Profit &amp; Loss Account'!C27:E27)</f>
@@ -29503,7 +29547,7 @@
     <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="195"/>
       <c r="B19" s="195" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C19" s="200" t="n">
         <f aca="false">SUM('Profit &amp; Loss Account'!C28:E28)</f>
@@ -29531,7 +29575,7 @@
     <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="195"/>
       <c r="B20" s="195" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C20" s="200" t="n">
         <f aca="false">SUM('Profit &amp; Loss Account'!C29:E29)</f>
@@ -29559,7 +29603,7 @@
     <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="195"/>
       <c r="B21" s="195" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C21" s="200" t="n">
         <f aca="false">SUM('Profit &amp; Loss Account'!C30:E30)</f>
@@ -29587,7 +29631,7 @@
     <row r="22" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="195"/>
       <c r="B22" s="195" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C22" s="200" t="n">
         <f aca="false">SUM('Profit &amp; Loss Account'!C32:E32)</f>
@@ -29626,7 +29670,7 @@
     <row r="24" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="195"/>
       <c r="B24" s="195" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C24" s="200" t="n">
         <f aca="false">SUM('Profit &amp; Loss Account'!C15:E15)</f>
@@ -29654,7 +29698,7 @@
     <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="195"/>
       <c r="B25" s="195" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C25" s="200" t="n">
         <f aca="false">SUM('Profit &amp; Loss Account'!C49:E49)</f>
@@ -29682,7 +29726,7 @@
     <row r="26" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="195"/>
       <c r="B26" s="195" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C26" s="200" t="n">
         <f aca="false">SUM('Profit &amp; Loss Account'!C33:E34)</f>
@@ -29732,7 +29776,7 @@
     <row r="29" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="195"/>
       <c r="B29" s="202" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C29" s="203" t="n">
         <f aca="false">SUM(C7,C12,C13,C14,C15,C16,C17,C18,C19,C20,C21,C22,C24,C26)</f>
@@ -29828,7 +29872,7 @@
     <row r="36" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="195"/>
       <c r="B36" s="195" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C36" s="200" t="n">
         <f aca="false">C7*$I$36</f>
@@ -29851,7 +29895,7 @@
         <v>269.4</v>
       </c>
       <c r="H36" s="195" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="I36" s="195" t="n">
         <v>0.02</v>
@@ -29860,7 +29904,7 @@
     <row r="37" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="195"/>
       <c r="B37" s="195" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C37" s="200" t="n">
         <f aca="false">C24*$I$37</f>
@@ -29883,7 +29927,7 @@
         <v>200</v>
       </c>
       <c r="H37" s="195" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="I37" s="195" t="n">
         <v>0.03</v>
@@ -29892,7 +29936,7 @@
     <row r="38" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="195"/>
       <c r="B38" s="195" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C38" s="200" t="n">
         <f aca="false">C12*$I$38</f>
@@ -29915,7 +29959,7 @@
         <v>3709.42933333333</v>
       </c>
       <c r="H38" s="195" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="I38" s="195" t="n">
         <v>0.04</v>
@@ -29924,7 +29968,7 @@
     <row r="39" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="195"/>
       <c r="B39" s="195" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C39" s="200" t="n">
         <f aca="false">C17*$I$39</f>
@@ -29947,7 +29991,7 @@
         <v>1996.0625</v>
       </c>
       <c r="H39" s="195" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="I39" s="195" t="n">
         <v>0.25</v>
@@ -29956,7 +30000,7 @@
     <row r="40" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="195"/>
       <c r="B40" s="195" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C40" s="200" t="n">
         <f aca="false">C13*$I$40</f>
@@ -29979,7 +30023,7 @@
         <v>660</v>
       </c>
       <c r="H40" s="195" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="I40" s="195" t="n">
         <v>0.05</v>
@@ -29988,7 +30032,7 @@
     <row r="41" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="195"/>
       <c r="B41" s="195" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C41" s="200" t="n">
         <f aca="false">C14*$I$41</f>
@@ -30011,7 +30055,7 @@
         <v>57</v>
       </c>
       <c r="H41" s="195" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="I41" s="195" t="n">
         <v>0.06</v>
@@ -30020,7 +30064,7 @@
     <row r="42" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="195"/>
       <c r="B42" s="195" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C42" s="200" t="n">
         <f aca="false">C15*$I$42</f>
@@ -30043,7 +30087,7 @@
         <v>212.45</v>
       </c>
       <c r="H42" s="195" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="I42" s="195" t="n">
         <v>0.07</v>
@@ -30052,7 +30096,7 @@
     <row r="43" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="195"/>
       <c r="B43" s="195" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C43" s="200" t="n">
         <f aca="false">C18*$I$43</f>
@@ -30075,7 +30119,7 @@
         <v>327.333333333333</v>
       </c>
       <c r="H43" s="195" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="I43" s="195" t="n">
         <v>0.08</v>
@@ -30084,7 +30128,7 @@
     <row r="44" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="195"/>
       <c r="B44" s="195" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C44" s="200" t="n">
         <f aca="false">C25</f>
@@ -30107,14 +30151,14 @@
         <v>291.666666666667</v>
       </c>
       <c r="H44" s="195" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="I44" s="195"/>
     </row>
     <row r="45" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="195"/>
       <c r="B45" s="195" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C45" s="200" t="n">
         <f aca="false">C21*$I$45</f>
@@ -30137,7 +30181,7 @@
         <v>0</v>
       </c>
       <c r="H45" s="195" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="I45" s="195" t="n">
         <v>0.09</v>
@@ -30146,7 +30190,7 @@
     <row r="46" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="195"/>
       <c r="B46" s="195" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C46" s="200" t="n">
         <f aca="false">C16*$I$46</f>
@@ -30169,7 +30213,7 @@
         <v>390</v>
       </c>
       <c r="H46" s="195" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="I46" s="195" t="n">
         <v>0.1</v>
@@ -30178,7 +30222,7 @@
     <row r="47" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="195"/>
       <c r="B47" s="195" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C47" s="200" t="n">
         <f aca="false">C20*$I$47</f>
@@ -30201,7 +30245,7 @@
         <v>-33</v>
       </c>
       <c r="H47" s="195" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="I47" s="195" t="n">
         <v>0.11</v>
@@ -30210,7 +30254,7 @@
     <row r="48" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="195"/>
       <c r="B48" s="195" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C48" s="200" t="n">
         <f aca="false">C19*$I$48</f>
@@ -30233,7 +30277,7 @@
         <v>831</v>
       </c>
       <c r="H48" s="195" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="I48" s="195" t="n">
         <v>0.12</v>
@@ -30242,7 +30286,7 @@
     <row r="49" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="195"/>
       <c r="B49" s="195" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C49" s="200" t="n">
         <f aca="false">SUM('Profit &amp; Loss Account'!C34:E34)</f>
@@ -30265,14 +30309,14 @@
         <v>20865</v>
       </c>
       <c r="H49" s="195" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="I49" s="195"/>
     </row>
     <row r="50" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="195"/>
       <c r="B50" s="195" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C50" s="200" t="n">
         <f aca="false">C22*$I$50</f>
@@ -30295,7 +30339,7 @@
         <v>420.116666666666</v>
       </c>
       <c r="H50" s="195" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="I50" s="195" t="n">
         <v>0.13</v>
@@ -30368,14 +30412,14 @@
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="211"/>
       <c r="B2" s="215" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C2" s="216" t="str">
         <f aca="false">Admin!L2</f>
         <v>2026-27</v>
       </c>
       <c r="D2" s="217" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="E2" s="217"/>
       <c r="F2" s="217"/>
@@ -30402,13 +30446,13 @@
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="211"/>
       <c r="B5" s="222" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C5" s="222"/>
       <c r="D5" s="222"/>
       <c r="E5" s="223" t="n">
         <f aca="false">'SE Full'!O210</f>
-        <v>125308.8085</v>
+        <v>124284.150965753</v>
       </c>
       <c r="F5" s="214"/>
       <c r="G5" s="218"/>
@@ -30417,7 +30461,7 @@
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="211"/>
       <c r="B6" s="220" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C6" s="220" t="str">
         <f aca="false">C2</f>
@@ -30426,7 +30470,7 @@
       <c r="D6" s="225"/>
       <c r="E6" s="218" t="n">
         <f aca="false">IF(E5&lt;=0,0,MAX(0,Admin!N$4-MAX(0,E5-Admin!N$5)/2))</f>
-        <v>0</v>
+        <v>427.924517123494</v>
       </c>
       <c r="F6" s="214"/>
       <c r="G6" s="218"/>
@@ -30435,13 +30479,13 @@
     <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="211"/>
       <c r="B7" s="222" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C7" s="222"/>
       <c r="D7" s="222"/>
       <c r="E7" s="223" t="n">
         <f aca="false">IF((E5&gt;E6),(E5-E6),0)</f>
-        <v>125308.8085</v>
+        <v>123856.22644863</v>
       </c>
       <c r="F7" s="214"/>
       <c r="G7" s="218"/>
@@ -30450,7 +30494,7 @@
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="211"/>
       <c r="B8" s="220" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C8" s="220" t="n">
         <f aca="false">Admin!N$11</f>
@@ -30472,7 +30516,7 @@
     <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="211"/>
       <c r="B9" s="220" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C9" s="220" t="n">
         <f aca="false">Admin!M$11</f>
@@ -30484,7 +30528,7 @@
       </c>
       <c r="E9" s="213" t="n">
         <f aca="false">IF(E7&gt;C9,(MIN(E7,C10)-C9)*D9,0)</f>
-        <v>34976</v>
+        <v>34462.4905794518</v>
       </c>
       <c r="F9" s="214"/>
       <c r="G9" s="218"/>
@@ -30493,7 +30537,7 @@
     <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="211"/>
       <c r="B10" s="220" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C10" s="220" t="n">
         <f aca="false">Admin!N$13</f>
@@ -30505,7 +30549,7 @@
       </c>
       <c r="E10" s="213" t="n">
         <f aca="false">IF(E7&gt;C10,(E7-C10)*D10,0)</f>
-        <v>75.9638249998163</v>
+        <v>0</v>
       </c>
       <c r="F10" s="214"/>
       <c r="G10" s="218"/>
@@ -30514,13 +30558,13 @@
     <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="211"/>
       <c r="B11" s="228" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C11" s="229"/>
       <c r="D11" s="230"/>
       <c r="E11" s="231" t="n">
         <f aca="false">SUM(E8:E10)</f>
-        <v>42591.9638249998</v>
+        <v>42002.4905794518</v>
       </c>
       <c r="F11" s="232"/>
       <c r="G11" s="233"/>
@@ -30529,7 +30573,7 @@
     <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="211"/>
       <c r="B12" s="220" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C12" s="220"/>
       <c r="D12" s="234"/>
@@ -30544,7 +30588,7 @@
     <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="211"/>
       <c r="B13" s="235" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C13" s="236" t="n">
         <f aca="false">Admin!B21</f>
@@ -30569,7 +30613,7 @@
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="211"/>
       <c r="B15" s="239" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C15" s="239"/>
       <c r="D15" s="226" t="n">
@@ -30587,7 +30631,7 @@
     <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="211"/>
       <c r="B16" s="239" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C16" s="239"/>
       <c r="D16" s="226" t="n">
@@ -30596,7 +30640,7 @@
       </c>
       <c r="E16" s="240" t="n">
         <f aca="false">IF((E5&gt;Admin!N$23),((E5-Admin!N$23)*D16),0)</f>
-        <v>1500.77616999999</v>
+        <v>1480.28301931506</v>
       </c>
       <c r="F16" s="214"/>
       <c r="G16" s="233"/>
@@ -30615,13 +30659,13 @@
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="211"/>
       <c r="B18" s="241" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C18" s="241"/>
       <c r="D18" s="237"/>
       <c r="E18" s="231" t="n">
         <f aca="false">SUM(E11:E17)</f>
-        <v>46354.7399949998</v>
+        <v>45744.7735987669</v>
       </c>
       <c r="F18" s="214"/>
       <c r="G18" s="218"/>
@@ -30648,11 +30692,11 @@
     <row r="21" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="211"/>
       <c r="B21" s="228" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C21" s="243"/>
       <c r="D21" s="244" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="E21" s="244"/>
       <c r="F21" s="244"/>
@@ -30672,10 +30716,10 @@
       <c r="B23" s="220"/>
       <c r="C23" s="220"/>
       <c r="D23" s="246" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="E23" s="247" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="F23" s="248"/>
       <c r="G23" s="218"/>
@@ -31192,18 +31236,18 @@
     <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="211"/>
       <c r="B25" s="220" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="C25" s="250" t="str">
         <f aca="false">Admin!B24</f>
         <v>2027-28</v>
       </c>
       <c r="D25" s="251" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="E25" s="240" t="n">
         <f aca="false">E18</f>
-        <v>46354.7399949998</v>
+        <v>45744.7735987669</v>
       </c>
       <c r="F25" s="214"/>
       <c r="G25" s="218"/>
@@ -31211,7 +31255,7 @@
     <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="211"/>
       <c r="B26" s="220" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C26" s="220"/>
       <c r="D26" s="252" t="n">
@@ -31220,7 +31264,7 @@
       </c>
       <c r="E26" s="223" t="n">
         <f aca="false">E25/2</f>
-        <v>23177.3699974999</v>
+        <v>22872.3867993834</v>
       </c>
       <c r="F26" s="214"/>
       <c r="G26" s="218"/>
@@ -31228,7 +31272,7 @@
     <row r="27" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="211"/>
       <c r="B27" s="220" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C27" s="220"/>
       <c r="D27" s="252" t="n">
@@ -31237,7 +31281,7 @@
       </c>
       <c r="E27" s="223" t="n">
         <f aca="false">E25/2</f>
-        <v>23177.3699974999</v>
+        <v>22872.3867993834</v>
       </c>
       <c r="F27" s="214"/>
       <c r="G27" s="218"/>
@@ -31254,7 +31298,7 @@
     <row r="29" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="211"/>
       <c r="B29" s="253" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C29" s="254"/>
       <c r="D29" s="237"/>
@@ -31265,7 +31309,7 @@
     <row r="30" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="211"/>
       <c r="B30" s="255" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C30" s="255"/>
       <c r="D30" s="211"/>
@@ -31276,7 +31320,7 @@
     <row r="31" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="211"/>
       <c r="B31" s="258" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C31" s="258"/>
       <c r="D31" s="259"/>
@@ -31287,7 +31331,7 @@
     <row r="32" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="211"/>
       <c r="B32" s="260" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C32" s="258"/>
       <c r="D32" s="259"/>
@@ -31298,7 +31342,7 @@
     <row r="33" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="211"/>
       <c r="B33" s="254" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="C33" s="254"/>
       <c r="D33" s="259"/>
@@ -31309,7 +31353,7 @@
     <row r="34" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="211"/>
       <c r="B34" s="254" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C34" s="254"/>
       <c r="D34" s="259"/>
@@ -31320,7 +31364,7 @@
     <row r="35" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="211"/>
       <c r="B35" s="254" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C35" s="254"/>
       <c r="D35" s="259"/>
@@ -31395,32 +31439,32 @@
     <row r="2" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="267"/>
       <c r="B2" s="268" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C2" s="269" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="D2" s="269" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E2" s="269" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="F2" s="269" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="G2" s="269" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="H2" s="269" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="I2" s="269" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="J2" s="270"/>
       <c r="K2" s="268" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="L2" s="271"/>
       <c r="M2" s="272"/>
@@ -31672,7 +31716,7 @@
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="267"/>
       <c r="B3" s="273" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C3" s="273"/>
       <c r="D3" s="274"/>
@@ -31966,7 +32010,7 @@
       </c>
       <c r="J4" s="158"/>
       <c r="K4" s="278" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="L4" s="164"/>
     </row>
@@ -32120,7 +32164,7 @@
       </c>
       <c r="J8" s="158"/>
       <c r="K8" s="278" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="L8" s="164"/>
     </row>
@@ -32472,7 +32516,7 @@
       <c r="F1" s="287"/>
       <c r="G1" s="287"/>
       <c r="H1" s="288" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="I1" s="288"/>
       <c r="J1" s="288"/>
@@ -32480,7 +32524,7 @@
       <c r="L1" s="288"/>
       <c r="M1" s="287"/>
       <c r="N1" s="288" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="O1" s="288"/>
       <c r="P1" s="288"/>
@@ -32488,7 +32532,7 @@
       <c r="R1" s="288"/>
       <c r="S1" s="287"/>
       <c r="T1" s="288" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="U1" s="288"/>
       <c r="V1" s="288"/>
@@ -32508,63 +32552,63 @@
     <row r="2" customFormat="false" ht="32.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="292"/>
       <c r="B2" s="293" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C2" s="294"/>
       <c r="D2" s="295" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="E2" s="296"/>
       <c r="F2" s="295" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="G2" s="296"/>
       <c r="H2" s="297" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="I2" s="296"/>
       <c r="J2" s="295" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="K2" s="296"/>
       <c r="L2" s="295" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="M2" s="296"/>
       <c r="N2" s="297" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="O2" s="296"/>
       <c r="P2" s="295" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="Q2" s="296"/>
       <c r="R2" s="295" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="S2" s="296"/>
       <c r="T2" s="297" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="U2" s="296"/>
       <c r="V2" s="295" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="W2" s="296"/>
       <c r="X2" s="298" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="Y2" s="299"/>
       <c r="Z2" s="295" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="AA2" s="296"/>
       <c r="AB2" s="295" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="AC2" s="300"/>
       <c r="AD2" s="301" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="AE2" s="301"/>
       <c r="AF2" s="301"/>
@@ -32825,7 +32869,7 @@
       <c r="AB3" s="305"/>
       <c r="AC3" s="164"/>
       <c r="AD3" s="309" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="AE3" s="309"/>
       <c r="AF3" s="309"/>
@@ -32835,7 +32879,7 @@
     <row r="4" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="276"/>
       <c r="B4" s="310" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C4" s="310"/>
       <c r="D4" s="310"/>
@@ -33215,7 +33259,7 @@
       <c r="AB11" s="177"/>
       <c r="AC11" s="164"/>
       <c r="AD11" s="309" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="AE11" s="309"/>
       <c r="AF11" s="309"/>
@@ -33445,7 +33489,7 @@
       <c r="AB15" s="177"/>
       <c r="AC15" s="164"/>
       <c r="AD15" s="309" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="AE15" s="309"/>
       <c r="AF15" s="309"/>
@@ -33675,7 +33719,7 @@
       <c r="AB19" s="177"/>
       <c r="AC19" s="164"/>
       <c r="AD19" s="309" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="AE19" s="309"/>
       <c r="AF19" s="309"/>
@@ -33905,7 +33949,7 @@
       <c r="AB23" s="177"/>
       <c r="AC23" s="164"/>
       <c r="AD23" s="309" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="AE23" s="309"/>
       <c r="AF23" s="309"/>
@@ -34213,7 +34257,7 @@
       </c>
       <c r="AC28" s="164"/>
       <c r="AD28" s="309" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="AE28" s="309"/>
       <c r="AF28" s="309"/>
@@ -34431,10 +34475,10 @@
     <row r="2" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="158"/>
       <c r="B2" s="330" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C2" s="161" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D2" s="162" t="n">
         <f aca="false">Admin!B5</f>
@@ -34554,7 +34598,7 @@
     <row r="5" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="178"/>
       <c r="B5" s="332" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C5" s="170" t="n">
         <f aca="false">SUM(D5:O5)</f>
@@ -35113,7 +35157,7 @@
     <row r="7" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="158"/>
       <c r="B7" s="334" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C7" s="170" t="n">
         <f aca="false">SUM(D7:O7)</f>
@@ -35190,7 +35234,7 @@
     <row r="9" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="178"/>
       <c r="B9" s="333" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C9" s="170" t="n">
         <f aca="false">SUM(D9:O9)</f>
@@ -35749,7 +35793,7 @@
     <row r="11" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="178"/>
       <c r="B11" s="332" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C11" s="170" t="n">
         <f aca="false">SUM(D11:O11)</f>
@@ -36308,7 +36352,7 @@
     <row r="13" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="158"/>
       <c r="B13" s="333" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C13" s="170" t="n">
         <f aca="false">SUM(D13:O13)</f>
@@ -36385,7 +36429,7 @@
     <row r="15" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="158"/>
       <c r="B15" s="332" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C15" s="170" t="n">
         <f aca="false">SUM(D15:O15)</f>
@@ -36444,7 +36488,7 @@
     <row r="16" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="158"/>
       <c r="B16" s="334" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C16" s="170" t="n">
         <f aca="false">SUM(D16:O16)</f>
@@ -36503,7 +36547,7 @@
     <row r="17" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="158"/>
       <c r="B17" s="335" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C17" s="170" t="n">
         <f aca="false">SUM(D17:O17)</f>
@@ -36580,10 +36624,10 @@
     <row r="19" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="158"/>
       <c r="B19" s="337" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C19" s="161" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D19" s="162" t="n">
         <f aca="false">D2</f>
@@ -36716,7 +36760,7 @@
     <row r="22" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="178"/>
       <c r="B22" s="332" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C22" s="170" t="n">
         <f aca="false">SUM(D22:O22)</f>
@@ -37275,7 +37319,7 @@
     <row r="24" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="158"/>
       <c r="B24" s="334" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C24" s="170" t="n">
         <f aca="false">SUM(D24:O24)</f>
@@ -37352,7 +37396,7 @@
     <row r="26" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="178"/>
       <c r="B26" s="333" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C26" s="170" t="n">
         <f aca="false">SUM(D26:O26)</f>
@@ -37911,7 +37955,7 @@
     <row r="28" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="178"/>
       <c r="B28" s="332" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C28" s="170" t="n">
         <f aca="false">SUM(D28:O28)</f>
@@ -38470,7 +38514,7 @@
     <row r="30" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="158"/>
       <c r="B30" s="333" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C30" s="170" t="n">
         <f aca="false">SUM(D30:O30)</f>
@@ -38547,7 +38591,7 @@
     <row r="32" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="158"/>
       <c r="B32" s="332" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C32" s="170" t="n">
         <f aca="false">SUM(D32:O32)</f>
@@ -38606,7 +38650,7 @@
     <row r="33" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="158"/>
       <c r="B33" s="334" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C33" s="170" t="n">
         <f aca="false">SUM(D33:O33)</f>
@@ -38665,7 +38709,7 @@
     <row r="34" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="158"/>
       <c r="B34" s="335" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C34" s="170" t="n">
         <f aca="false">SUM(D34:O34)</f>
@@ -38742,7 +38786,7 @@
     <row r="36" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="158"/>
       <c r="B36" s="338" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C36" s="338"/>
       <c r="D36" s="158"/>
@@ -38762,7 +38806,7 @@
     <row r="37" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="158"/>
       <c r="B37" s="169" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="C37" s="339" t="n">
         <f aca="false">'Profit &amp; Loss Account'!B33+'Profit &amp; Loss Account'!B34</f>
@@ -38785,7 +38829,7 @@
     <row r="38" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="158"/>
       <c r="B38" s="169" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="C38" s="339" t="n">
         <f aca="false">[1]Schedule!$Q$1+[1]Schedule!$R$1+[1]Schedule!$AC$1+[1]Schedule!$Y$1-[1]Schedule!$Z$1</f>
@@ -38808,7 +38852,7 @@
     <row r="39" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="158"/>
       <c r="B39" s="169" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C39" s="339" t="n">
         <f aca="false">C34+C37-C38</f>
@@ -38831,7 +38875,7 @@
     <row r="40" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="158"/>
       <c r="B40" s="182" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C40" s="339" t="n">
         <f aca="false">IF(C39&lt;=0,0,MAX(0,Admin!N$4-MAX(0,C39-Admin!N$5)/2))</f>
@@ -38854,7 +38898,7 @@
     <row r="41" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="158"/>
       <c r="B41" s="182" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="C41" s="339" t="n">
         <f aca="false">IF((C39&gt;C40),(C39-C40),0)</f>
@@ -38877,7 +38921,7 @@
     <row r="42" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="158"/>
       <c r="B42" s="182" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C42" s="339" t="n">
         <f aca="false">IF((C41&gt;0),(IF((C41&lt;Admin!M$11),C41*Admin!N$6,Admin!M$11*Admin!N$6)),0)</f>
@@ -38900,7 +38944,7 @@
     <row r="43" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="158"/>
       <c r="B43" s="182" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C43" s="339" t="n">
         <f aca="false">IF(C41&gt;Admin!M$11,(MIN(C41,Admin!N$13)-Admin!M$11)*Admin!N$7,0)</f>
@@ -38923,7 +38967,7 @@
     <row r="44" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="158"/>
       <c r="B44" s="182" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="C44" s="339" t="n">
         <f aca="false">IF(C41&gt;Admin!N$13,(C41-Admin!N$13)*Admin!N$8,0)</f>
@@ -38946,7 +38990,7 @@
     <row r="45" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="158"/>
       <c r="B45" s="182" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C45" s="339" t="n">
         <f aca="false">IF(C39&gt;Admin!N$20,IF(C39&lt;Admin!N$23,(C39-Admin!N$20)*Admin!L$20,(Admin!N$23-Admin!N$20)*Admin!L$20),0)+IF(C39&gt;Admin!N$23,(C39-Admin!N$23)*Admin!L$23,0)</f>
@@ -38969,7 +39013,7 @@
     <row r="46" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="158"/>
       <c r="B46" s="182" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="C46" s="341" t="n">
         <f aca="false">C42+C43+C44+C45</f>

</xml_diff>